<commit_message>
📊 Precios actualizados 2026-05-26
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -206,6 +206,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -220,9 +224,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -319,6 +320,1140 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Evolución del precio medio diario</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'📊 Media diaria'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
+              <a:solidFill>
+                <a:srgbClr val="2980B9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'📊 Media diaria'!$A$3:$A$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'📊 Media diaria'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
+              <a:solidFill>
+                <a:srgbClr val="8E44AD"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'📊 Media diaria'!$A$3:$A$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'📊 Media diaria'!D2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
+              <a:solidFill>
+                <a:srgbClr val="27AE60"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'📊 Media diaria'!$A$3:$A$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fecha</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Precio (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sikaflex 522 — Evolución de precio por tienda</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Andorra Campers</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>Barna Campers</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <v>Madrid Camper 522</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Obelink 522</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fecha</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Precio (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sikaflex 554 — Evolución de precio por tienda</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Berger Camping 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>Intercut 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <v>Madrid Camper 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Obelink 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fecha</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Precio (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sikaflex 621 — Evolución de precio por tienda</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Plana Online 621</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>Toolstock 621</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fecha</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Precio (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10800000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10800000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10800000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -630,14 +1765,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 25/05/2026 16:11</t>
+          <t>Última actualización: 26/05/2026 14:52</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-25</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -659,11 +1794,11 @@
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Barna Campers</t>
+          <t>Obelink 522</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>11.5</v>
+        <v>10.99</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
@@ -674,11 +1809,11 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Andorra Campers</t>
+          <t>Barna Campers</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
@@ -699,7 +1834,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-25</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -771,7 +1906,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-25</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -838,7 +1973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -892,11 +2027,28 @@
         <v>13.4</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -906,34 +2058,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>SIKAFLEX 522 — Precio por tienda y fecha</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Andorra Campers</t>
         </is>
@@ -941,19 +2099,23 @@
       <c r="B3" s="19" t="n">
         <v>11.6</v>
       </c>
+      <c r="C3" s="19" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Barna Campers</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="21" t="n">
         <v>11.5</v>
       </c>
+      <c r="C4" s="21" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Madrid Camper 522</t>
         </is>
@@ -961,12 +2123,27 @@
       <c r="B5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="C5" s="19" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -976,34 +2153,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>SIKAFLEX 554 — Precio por tienda y fecha</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Berger Camping 554</t>
         </is>
@@ -1011,19 +2194,25 @@
       <c r="B3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="C3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Intercut 554</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="21" t="n">
         <v>16.84</v>
       </c>
+      <c r="C4" s="21" t="n">
+        <v>16.84</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Madrid Camper 554</t>
         </is>
@@ -1031,22 +2220,29 @@
       <c r="B5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="C5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Obelink 554</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="C6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1056,34 +2252,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>SIKAFLEX 621 — Precio por tienda y fecha</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
@@ -1091,22 +2293,29 @@
       <c r="B3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="C3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="21" t="n">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1116,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1127,7 +2336,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="31" t="inlineStr">
         <is>
           <t>HISTÓRICO COMPLETO DE PRECIOS — SIKAFLEX</t>
         </is>
@@ -1161,17 +2370,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="31" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B3" s="31" t="inlineStr">
+      <c r="B3" s="32" t="inlineStr">
         <is>
           <t>522</t>
         </is>
       </c>
-      <c r="C3" s="31" t="inlineStr">
+      <c r="C3" s="32" t="inlineStr">
         <is>
           <t>Andorra Campers</t>
         </is>
@@ -1179,49 +2388,49 @@
       <c r="D3" s="19" t="n">
         <v>11.6</v>
       </c>
-      <c r="E3" s="31" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
         <is>
           <t>https://www.andorracampers.com/es/sikaflex-522-blanca_3485_342.html</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>522</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>Barna Campers</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D4" s="21" t="n">
         <v>11.5</v>
       </c>
-      <c r="E4" s="32" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
         <is>
           <t>522</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Madrid Camper 522</t>
         </is>
@@ -1229,49 +2438,49 @@
       <c r="D5" s="19" t="n">
         <v>12.4</v>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="32" t="inlineStr">
         <is>
           <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B6" s="32" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>554</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>Intercut 554</t>
         </is>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="21" t="n">
         <v>16.84</v>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>554</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>Obelink 554</t>
         </is>
@@ -1279,49 +2488,49 @@
       <c r="D7" s="19" t="n">
         <v>17.99</v>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="32" t="inlineStr">
         <is>
           <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>554</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>Berger Camping 554</t>
         </is>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="21" t="n">
         <v>21.75</v>
       </c>
-      <c r="E8" s="32" t="inlineStr">
+      <c r="E8" s="33" t="inlineStr">
         <is>
           <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>554</t>
         </is>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>Madrid Camper 554</t>
         </is>
@@ -1329,49 +2538,49 @@
       <c r="D9" s="19" t="n">
         <v>18.87</v>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="32" t="inlineStr">
         <is>
           <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>621</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="E10" s="32" t="inlineStr">
+      <c r="E10" s="33" t="inlineStr">
         <is>
           <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>621</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
@@ -1379,9 +2588,484 @@
       <c r="D11" s="19" t="n">
         <v>11.8</v>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="32" t="inlineStr">
         <is>
           <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E28" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-05-27
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -174,15 +174,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$4</f>
+              <f>'📊 Media diaria'!$A$3:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$4</f>
+              <f>'📊 Media diaria'!$B$3:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$4</f>
+              <f>'📊 Media diaria'!$A$3:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$4</f>
+              <f>'📊 Media diaria'!$C$3:$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$4</f>
+              <f>'📊 Media diaria'!$A$3:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$4</f>
+              <f>'📊 Media diaria'!$D$3:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
@@ -569,6 +569,33 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -587,18 +614,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$3</f>
+              <f>'🔵 Sikaflex 522'!$D$3</f>
             </numRef>
           </val>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -614,42 +641,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'🔵 Sikaflex 522'!$B$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <v>Barna Campers</v>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -671,12 +668,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -684,7 +681,7 @@
           <idx val="5"/>
           <order val="5"/>
           <tx>
-            <v>Madrid Camper 522</v>
+            <v>Barna Campers</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -701,12 +698,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -728,18 +725,129 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <v>Madrid Camper 522</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -758,12 +866,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$C$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -872,7 +980,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
@@ -884,6 +992,33 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -902,18 +1037,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$3</f>
+              <f>'🟣 Sikaflex 554'!$D$3</f>
             </numRef>
           </val>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -929,42 +1064,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'🟣 Sikaflex 554'!$B$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <v>Intercut 554</v>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -986,12 +1091,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -999,7 +1104,7 @@
           <idx val="5"/>
           <order val="5"/>
           <tx>
-            <v>Madrid Camper 554</v>
+            <v>Intercut 554</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1016,12 +1121,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1043,18 +1148,129 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <v>Madrid Camper 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -1073,12 +1289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$C$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1187,7 +1403,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
@@ -1199,6 +1415,33 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -1217,18 +1460,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$C$3</f>
+              <f>'🟢 Sikaflex 621'!$D$3</f>
             </numRef>
           </val>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1244,7 +1487,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
@@ -1254,8 +1497,35 @@
           </val>
         </ser>
         <ser>
-          <idx val="3"/>
-          <order val="3"/>
+          <idx val="4"/>
+          <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -1274,12 +1544,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$C$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1354,7 +1624,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -1745,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1765,14 +2035,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 26/05/2026 18:11</t>
+          <t>Última actualización: 27/05/2026 06:24</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-26</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -1815,141 +2085,121 @@
       <c r="B7" s="8" t="n">
         <v>11.5</v>
       </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 522</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>17.99</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Obelink 554</t>
+          <t>Berger Camping 554</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>17.99</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 554</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>18.87</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Berger Camping 554</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
         <v>21.75</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B17" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B18" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -1959,9 +2209,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1973,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2040,6 +2290,22 @@
         <v>18.86</v>
       </c>
       <c r="D4" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D5" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -2058,12 +2324,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2089,6 +2356,11 @@
           <t>2026-05-26</t>
         </is>
       </c>
+      <c r="D2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2100,6 +2372,7 @@
         <v>11.6</v>
       </c>
       <c r="C3" s="19" t="n"/>
+      <c r="D3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2113,6 +2386,9 @@
       <c r="C4" s="21" t="n">
         <v>11.5</v>
       </c>
+      <c r="D4" s="21" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -2126,6 +2402,7 @@
       <c r="C5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="D5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2137,10 +2414,13 @@
       <c r="C6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="D6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2153,12 +2433,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2184,6 +2465,11 @@
           <t>2026-05-26</t>
         </is>
       </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2197,6 +2483,9 @@
       <c r="C3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="D3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2210,6 +2499,9 @@
       <c r="C4" s="21" t="n">
         <v>16.84</v>
       </c>
+      <c r="D4" s="21" t="n">
+        <v>16.84</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -2223,6 +2515,7 @@
       <c r="C5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="D5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2236,10 +2529,13 @@
       <c r="C6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="D6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2252,12 +2548,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2283,6 +2580,11 @@
           <t>2026-05-26</t>
         </is>
       </c>
+      <c r="D2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2296,6 +2598,9 @@
       <c r="C3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="D3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2309,10 +2614,13 @@
       <c r="C4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="D4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2325,7 +2633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3069,6 +3377,431 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E31" s="32" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B32" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C32" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E32" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E33" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E34" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C35" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E35" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B36" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C36" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E36" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E37" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C39" s="32" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E39" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B41" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C41" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E41" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E42" s="33" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B43" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C43" s="32" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D43" s="19" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E43" s="32" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B44" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E44" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B45" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C45" s="32" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D45" s="19" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E45" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B46" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D46" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E46" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B47" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C47" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E47" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-05-28
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$5</f>
+              <f>'📊 Media diaria'!$A$3:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$5</f>
+              <f>'📊 Media diaria'!$B$3:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$5</f>
+              <f>'📊 Media diaria'!$A$3:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$5</f>
+              <f>'📊 Media diaria'!$C$3:$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$5</f>
+              <f>'📊 Media diaria'!$A$3:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$5</f>
+              <f>'📊 Media diaria'!$D$3:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -596,6 +596,33 @@
         <ser>
           <idx val="2"/>
           <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -614,39 +641,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -668,21 +668,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="5"/>
           <order val="5"/>
-          <tx>
-            <v>Barna Campers</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -698,12 +695,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -725,47 +722,20 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
           <tx>
-            <v>Madrid Camper 522</v>
+            <v>Barna Campers</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -782,12 +752,39 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -809,12 +806,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -836,18 +833,129 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <tx>
+            <v>Madrid Camper 522</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -866,12 +974,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$D$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -980,7 +1088,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -1007,7 +1115,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -1019,6 +1127,33 @@
         <ser>
           <idx val="2"/>
           <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1037,39 +1172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -1091,21 +1199,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="5"/>
           <order val="5"/>
-          <tx>
-            <v>Intercut 554</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1121,12 +1226,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1148,47 +1253,20 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
           <tx>
-            <v>Madrid Camper 554</v>
+            <v>Intercut 554</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1205,12 +1283,39 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1232,12 +1337,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1259,18 +1364,129 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <tx>
+            <v>Madrid Camper 554</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -1289,12 +1505,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$D$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1403,7 +1619,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -1430,7 +1646,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
@@ -1442,6 +1658,33 @@
         <ser>
           <idx val="2"/>
           <order val="2"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -1460,39 +1703,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$D$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -1514,18 +1730,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="5"/>
           <order val="5"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -1544,12 +1814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$D$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1624,7 +1894,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>8</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -2035,14 +2305,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 27/05/2026 08:24</t>
+          <t>Última actualización: 28/05/2026 10:57</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-27</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2364,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-27</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2426,7 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-27</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2306,6 +2576,22 @@
         <v>18.86</v>
       </c>
       <c r="D5" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D6" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -2324,13 +2610,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2361,6 +2648,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="E2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2373,6 +2665,7 @@
       </c>
       <c r="C3" s="19" t="n"/>
       <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2389,6 +2682,9 @@
       <c r="D4" s="21" t="n">
         <v>11.5</v>
       </c>
+      <c r="E4" s="21" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -2403,6 +2699,7 @@
         <v>12.4</v>
       </c>
       <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2417,10 +2714,13 @@
       <c r="D6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="E6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2433,13 +2733,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2470,6 +2771,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2486,6 +2792,9 @@
       <c r="D3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="E3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2502,6 +2811,9 @@
       <c r="D4" s="21" t="n">
         <v>16.84</v>
       </c>
+      <c r="E4" s="21" t="n">
+        <v>16.84</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -2516,6 +2828,7 @@
         <v>18.87</v>
       </c>
       <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2532,10 +2845,13 @@
       <c r="D6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="E6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2548,13 +2864,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2585,6 +2902,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="E2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2601,6 +2923,9 @@
       <c r="D3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="E3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2617,10 +2942,13 @@
       <c r="D4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="E4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2633,7 +2961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3827,6 +4155,456 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E49" s="32" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C50" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E50" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B51" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E51" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B52" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C52" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E52" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E53" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B54" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C54" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E54" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B55" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E55" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B56" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C56" s="33" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E56" s="33" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C57" s="32" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E57" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B58" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C58" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D58" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E58" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B59" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C59" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E59" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B60" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C60" s="33" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E60" s="33" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C61" s="32" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E61" s="32" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B62" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C62" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E62" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C63" s="32" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E63" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B64" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C64" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B65" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C65" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E65" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B66" s="33" t="inlineStr">
+        <is>
+          <t>SP101</t>
+        </is>
+      </c>
+      <c r="C66" s="33" t="inlineStr">
+        <is>
+          <t>ModregoHogar SP101</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E66" s="33" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/siliconas-y-masillas/instant-tack-sp101-cartucho-blanco.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-05-29
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -174,15 +174,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$6</f>
+              <f>'📊 Media diaria'!$A$3:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$6</f>
+              <f>'📊 Media diaria'!$B$3:$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$6</f>
+              <f>'📊 Media diaria'!$A$3:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$6</f>
+              <f>'📊 Media diaria'!$C$3:$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$6</f>
+              <f>'📊 Media diaria'!$A$3:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$6</f>
+              <f>'📊 Media diaria'!$D$3:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -623,6 +623,33 @@
         <ser>
           <idx val="3"/>
           <order val="3"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -641,39 +668,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$F$3</f>
             </numRef>
           </val>
         </ser>
@@ -695,12 +695,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -722,21 +722,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
-          <tx>
-            <v>Barna Campers</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -752,12 +749,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -779,18 +776,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <tx>
+            <v>Barna Campers</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -806,12 +806,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -833,21 +833,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
-          <tx>
-            <v>Madrid Camper 522</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -863,12 +860,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -890,12 +887,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -917,18 +914,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="14"/>
           <order val="14"/>
+          <tx>
+            <v>Madrid Camper 522</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -944,18 +944,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -974,12 +1082,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$E$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1088,7 +1196,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1115,7 +1223,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1142,7 +1250,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1154,6 +1262,33 @@
         <ser>
           <idx val="3"/>
           <order val="3"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1172,39 +1307,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$F$3</f>
             </numRef>
           </val>
         </ser>
@@ -1226,12 +1334,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1253,21 +1361,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
-          <tx>
-            <v>Intercut 554</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1283,12 +1388,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1310,18 +1415,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <tx>
+            <v>Intercut 554</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1337,12 +1445,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1364,21 +1472,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
-          <tx>
-            <v>Madrid Camper 554</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1394,12 +1499,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1421,12 +1526,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1448,18 +1553,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="14"/>
           <order val="14"/>
+          <tx>
+            <v>Madrid Camper 554</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1475,18 +1583,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -1505,12 +1721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$E$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1619,7 +1835,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1646,7 +1862,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1673,7 +1889,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
@@ -1685,6 +1901,33 @@
         <ser>
           <idx val="3"/>
           <order val="3"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -1703,39 +1946,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$E$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$F$3</f>
             </numRef>
           </val>
         </ser>
@@ -1757,12 +1973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1784,18 +2000,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -1814,12 +2084,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$E$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1894,7 +2164,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>8</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -2285,7 +2555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2305,14 +2575,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 28/05/2026 17:56</t>
+          <t>Última actualización: 29/05/2026 10:51</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-28</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2355,141 +2625,121 @@
       <c r="B7" s="8" t="n">
         <v>11.5</v>
       </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 522</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>17.99</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Obelink 554</t>
+          <t>Berger Camping 554</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>17.99</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 554</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>18.87</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Berger Camping 554</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
         <v>21.75</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B17" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B18" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -2499,9 +2749,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2513,7 +2763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2612,6 +2862,22 @@
         <v>18.86</v>
       </c>
       <c r="D6" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D7" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -2630,7 +2896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2638,6 +2904,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2673,6 +2940,11 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="F2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2686,6 +2958,7 @@
       <c r="C3" s="19" t="n"/>
       <c r="D3" s="19" t="n"/>
       <c r="E3" s="19" t="n"/>
+      <c r="F3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2703,6 +2976,9 @@
         <v>11.5</v>
       </c>
       <c r="E4" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F4" s="21" t="n">
         <v>11.5</v>
       </c>
     </row>
@@ -2722,6 +2998,7 @@
       <c r="E5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="F5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2739,10 +3016,13 @@
       <c r="E6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="F6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2755,7 +3035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2763,6 +3043,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2798,6 +3079,11 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2817,6 +3103,9 @@
       <c r="E3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="F3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2834,6 +3123,9 @@
         <v>16.84</v>
       </c>
       <c r="E4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="F4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -2853,6 +3145,7 @@
       <c r="E5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="F5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -2872,10 +3165,13 @@
       <c r="E6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="F6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2888,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2896,6 +3192,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2931,6 +3228,11 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="F2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2950,6 +3252,9 @@
       <c r="E3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="F3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2969,10 +3274,13 @@
       <c r="E4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="F4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2985,7 +3293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4679,6 +4987,431 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B69" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E69" s="32" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B70" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C70" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E70" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B71" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C72" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E72" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B74" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C74" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E74" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B75" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C75" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D75" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E75" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B76" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C76" s="33" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D76" s="21" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E76" s="33" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B77" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C77" s="32" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D77" s="19" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E77" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B78" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C78" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E78" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B80" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C80" s="33" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D80" s="21" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E80" s="33" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B82" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C82" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D82" s="21" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E82" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B83" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C83" s="32" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E83" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B84" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C84" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D84" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E84" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B85" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C85" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E85" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-05-30
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$7</f>
+              <f>'📊 Media diaria'!$A$3:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$7</f>
+              <f>'📊 Media diaria'!$B$3:$B$8</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$7</f>
+              <f>'📊 Media diaria'!$A$3:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$7</f>
+              <f>'📊 Media diaria'!$C$3:$C$8</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$7</f>
+              <f>'📊 Media diaria'!$A$3:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$7</f>
+              <f>'📊 Media diaria'!$D$3:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -650,6 +650,33 @@
         <ser>
           <idx val="4"/>
           <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -668,39 +695,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$F$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$G$3</f>
             </numRef>
           </val>
         </ser>
@@ -722,12 +722,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -749,12 +749,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -776,21 +776,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="9"/>
           <order val="9"/>
-          <tx>
-            <v>Barna Campers</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -806,12 +803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -833,18 +830,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <tx>
+            <v>Barna Campers</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -860,12 +860,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -887,12 +887,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -914,21 +914,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="14"/>
           <order val="14"/>
-          <tx>
-            <v>Madrid Camper 522</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -944,12 +941,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -971,12 +968,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -998,18 +995,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <tx>
+            <v>Madrid Camper 522</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1025,12 +1025,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1052,18 +1052,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="19"/>
           <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1082,12 +1190,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$F$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1196,7 +1304,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1223,7 +1331,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1250,7 +1358,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1277,7 +1385,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1289,6 +1397,33 @@
         <ser>
           <idx val="4"/>
           <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1307,39 +1442,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$F$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$G$3</f>
             </numRef>
           </val>
         </ser>
@@ -1361,12 +1469,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1388,12 +1496,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1415,21 +1523,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="9"/>
           <order val="9"/>
-          <tx>
-            <v>Intercut 554</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1445,12 +1550,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1472,18 +1577,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <tx>
+            <v>Intercut 554</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1499,12 +1607,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1526,12 +1634,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1553,21 +1661,18 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="14"/>
           <order val="14"/>
-          <tx>
-            <v>Madrid Camper 554</v>
-          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1583,12 +1688,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1610,12 +1715,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1637,18 +1742,21 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <tx>
+            <v>Madrid Camper 554</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1664,12 +1772,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1691,18 +1799,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="19"/>
           <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -1721,12 +1937,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$F$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1835,7 +2051,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1862,7 +2078,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1889,7 +2105,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1916,7 +2132,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
@@ -1928,6 +2144,33 @@
         <ser>
           <idx val="4"/>
           <order val="4"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -1946,39 +2189,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$F$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$G$3</f>
             </numRef>
           </val>
         </ser>
@@ -2000,12 +2216,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2027,12 +2243,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2054,18 +2270,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -2084,12 +2354,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$F$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2164,7 +2434,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -2575,14 +2845,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 29/05/2026 18:01</t>
+          <t>Última actualización: 30/05/2026 11:09</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-29</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2914,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-29</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2986,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-29</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2783,7 +3053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2898,6 +3168,22 @@
         <v>18.86</v>
       </c>
       <c r="D7" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D8" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -2916,7 +3202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2925,6 +3211,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2965,6 +3252,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
+      <c r="G2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -2979,6 +3271,7 @@
       <c r="D3" s="19" t="n"/>
       <c r="E3" s="19" t="n"/>
       <c r="F3" s="19" t="n"/>
+      <c r="G3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -2999,6 +3292,9 @@
         <v>11.5</v>
       </c>
       <c r="F4" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G4" s="21" t="n">
         <v>11.5</v>
       </c>
     </row>
@@ -3021,6 +3317,9 @@
       <c r="F5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="G5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3041,10 +3340,13 @@
       <c r="F6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="G6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3057,7 +3359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3066,6 +3368,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3106,6 +3409,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3128,6 +3436,9 @@
       <c r="F3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="G3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3148,6 +3459,9 @@
         <v>16.84</v>
       </c>
       <c r="F4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="G4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -3170,6 +3484,9 @@
       <c r="F5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="G5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3192,10 +3509,13 @@
       <c r="F6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="G6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3208,7 +3528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3217,6 +3537,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3257,6 +3578,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
+      <c r="G2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3279,6 +3605,9 @@
       <c r="F3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="G3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3301,10 +3630,13 @@
       <c r="F4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="G4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3317,7 +3649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5486,6 +5818,506 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B88" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C88" s="33" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D88" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E88" s="33" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B89" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C89" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E89" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C90" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D90" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E90" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C91" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E91" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B92" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C92" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D92" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E92" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C93" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E93" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B94" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C94" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D94" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E94" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C95" s="32" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E95" s="32" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B96" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C96" s="33" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E96" s="33" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C97" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E97" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B98" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C98" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D98" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E98" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B99" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C99" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E99" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B100" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C100" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D100" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E100" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B101" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C101" s="32" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E101" s="32" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B102" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C102" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D102" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E102" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B103" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C103" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E103" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B104" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C104" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D104" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E104" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B105" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C105" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D105" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E105" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B106" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C106" s="33" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D106" s="21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E106" s="33" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B107" s="32" t="inlineStr">
+        <is>
+          <t>SP101</t>
+        </is>
+      </c>
+      <c r="C107" s="32" t="inlineStr">
+        <is>
+          <t>ModregoHogar SP101</t>
+        </is>
+      </c>
+      <c r="D107" s="19" t="n">
+        <v>197</v>
+      </c>
+      <c r="E107" s="32" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/siliconas-y-masillas/instant-tack-sp101-cartucho-blanco.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-05-31
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$8</f>
+              <f>'📊 Media diaria'!$A$3:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$8</f>
+              <f>'📊 Media diaria'!$A$3:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$8</f>
+              <f>'📊 Media diaria'!$A$3:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -677,6 +677,33 @@
         <ser>
           <idx val="5"/>
           <order val="5"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -695,39 +722,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -749,12 +749,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -776,12 +776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -803,12 +803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -830,18 +830,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -860,66 +914,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -941,12 +941,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -968,12 +968,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -995,18 +995,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1025,93 +1106,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1133,12 +1133,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1160,18 +1160,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1190,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1304,7 +1412,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -1331,7 +1439,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -1358,7 +1466,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -1385,7 +1493,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -1412,7 +1520,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -1424,6 +1532,33 @@
         <ser>
           <idx val="5"/>
           <order val="5"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1442,39 +1577,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -1496,12 +1604,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1523,12 +1631,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1550,12 +1658,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1577,18 +1685,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -1607,66 +1769,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1688,12 +1796,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1715,12 +1823,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1742,18 +1850,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -1772,93 +1961,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1880,12 +1988,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1907,18 +2015,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -1937,12 +2153,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2051,7 +2267,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -2078,7 +2294,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -2105,7 +2321,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -2132,7 +2348,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -2159,7 +2375,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
             </numRef>
           </cat>
           <val>
@@ -2171,6 +2387,33 @@
         <ser>
           <idx val="5"/>
           <order val="5"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -2189,39 +2432,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -2243,12 +2459,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2270,12 +2486,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2297,12 +2513,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2324,18 +2540,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -2354,12 +2624,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$G$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2434,7 +2704,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -2845,14 +3115,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 30/05/2026 11:09</t>
+          <t>Última actualización: 31/05/2026 11:55</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-30</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -2914,7 +3184,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-30</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -2986,7 +3256,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-30</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3184,6 +3454,22 @@
         <v>18.86</v>
       </c>
       <c r="D8" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D9" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -3202,7 +3488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3212,6 +3498,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3255,6 +3542,11 @@
       <c r="G2" s="24" t="inlineStr">
         <is>
           <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="H2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -3272,6 +3564,7 @@
       <c r="E3" s="19" t="n"/>
       <c r="F3" s="19" t="n"/>
       <c r="G3" s="19" t="n"/>
+      <c r="H3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3295,6 +3588,9 @@
         <v>11.5</v>
       </c>
       <c r="G4" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H4" s="21" t="n">
         <v>11.5</v>
       </c>
     </row>
@@ -3320,6 +3616,9 @@
       <c r="G5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="H5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3343,10 +3642,13 @@
       <c r="G6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="H6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3359,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3369,6 +3671,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3414,6 +3717,11 @@
           <t>2026-05-30</t>
         </is>
       </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3439,6 +3747,9 @@
       <c r="G3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="H3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3462,6 +3773,9 @@
         <v>16.84</v>
       </c>
       <c r="G4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="H4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -3487,6 +3801,9 @@
       <c r="G5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="H5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3512,10 +3829,13 @@
       <c r="G6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="H6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3528,7 +3848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3538,6 +3858,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3583,6 +3904,11 @@
           <t>2026-05-30</t>
         </is>
       </c>
+      <c r="H2" s="30" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3608,6 +3934,9 @@
       <c r="G3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="H3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3633,10 +3962,13 @@
       <c r="G4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="H4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3649,7 +3981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6318,6 +6650,506 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B108" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C108" s="33" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D108" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E108" s="33" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B109" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C109" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D109" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E109" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B110" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C110" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D110" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E110" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C111" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D111" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E111" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B112" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C112" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D112" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E112" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B113" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C113" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E113" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B114" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C114" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D114" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E114" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B115" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C115" s="32" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D115" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E115" s="32" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B116" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C116" s="33" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D116" s="21" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E116" s="33" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B117" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C117" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D117" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E117" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B118" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C118" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D118" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E118" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B119" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C119" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D119" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E119" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B120" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C120" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D120" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E120" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B121" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C121" s="32" t="inlineStr">
+        <is>
+          <t>Esteba SF45</t>
+        </is>
+      </c>
+      <c r="D121" s="19" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E121" s="32" t="inlineStr">
+        <is>
+          <t>https://www.esteba.com/es/adhesivo-sellador-pu-soudaflex-45fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B122" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C122" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D122" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E122" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B123" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C123" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D123" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E123" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B124" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C124" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D124" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E124" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B125" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C125" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D125" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E125" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B126" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C126" s="33" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D126" s="21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E126" s="33" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B127" s="32" t="inlineStr">
+        <is>
+          <t>SP101</t>
+        </is>
+      </c>
+      <c r="C127" s="32" t="inlineStr">
+        <is>
+          <t>ModregoHogar SP101</t>
+        </is>
+      </c>
+      <c r="D127" s="19" t="n">
+        <v>328</v>
+      </c>
+      <c r="E127" s="32" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/siliconas-y-masillas/instant-tack-sp101-cartucho-blanco.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-01
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -174,15 +174,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$9</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$9</f>
+              <f>'📊 Media diaria'!$A$3:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$10</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$9</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$9</f>
+              <f>'📊 Media diaria'!$A$3:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$10</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$9</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$9</f>
+              <f>'📊 Media diaria'!$A$3:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -704,6 +704,33 @@
         <ser>
           <idx val="6"/>
           <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -722,39 +749,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -776,12 +776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -803,12 +803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -830,12 +830,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -857,12 +857,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -884,18 +884,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -914,66 +968,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -995,12 +995,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1022,12 +1022,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1049,12 +1049,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1076,18 +1076,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="20"/>
           <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1106,93 +1187,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="21"/>
-          <order val="21"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="22"/>
-          <order val="22"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="23"/>
-          <order val="23"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1214,12 +1214,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1241,12 +1241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1268,18 +1268,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="27"/>
           <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1298,12 +1406,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1412,7 +1520,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1439,7 +1547,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1466,7 +1574,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1493,7 +1601,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1520,7 +1628,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1547,7 +1655,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -1559,6 +1667,33 @@
         <ser>
           <idx val="6"/>
           <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1577,39 +1712,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -1631,12 +1739,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1658,12 +1766,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1685,12 +1793,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1712,12 +1820,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1739,18 +1847,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -1769,66 +1931,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1850,12 +1958,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1877,12 +1985,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1904,12 +2012,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1931,18 +2039,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="20"/>
           <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -1961,93 +2150,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="21"/>
-          <order val="21"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="22"/>
-          <order val="22"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="23"/>
-          <order val="23"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -2069,12 +2177,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -2096,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -2123,18 +2231,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="27"/>
           <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -2153,12 +2369,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2267,7 +2483,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2294,7 +2510,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2321,7 +2537,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2348,7 +2564,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2375,7 +2591,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2402,7 +2618,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
             </numRef>
           </cat>
           <val>
@@ -2414,6 +2630,33 @@
         <ser>
           <idx val="6"/>
           <order val="6"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -2432,39 +2675,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -2486,12 +2702,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2513,12 +2729,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2540,12 +2756,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2567,12 +2783,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2594,18 +2810,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -2624,12 +2894,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$H$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2704,7 +2974,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>12</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -3095,7 +3365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3115,14 +3385,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 31/05/2026 11:55</t>
+          <t>Última actualización: 01/06/2026 10:12</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-05-31</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3165,141 +3435,121 @@
       <c r="B7" s="8" t="n">
         <v>11.5</v>
       </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 522</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>17.99</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Obelink 554</t>
+          <t>Berger Camping 554</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>17.99</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 554</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>18.87</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Berger Camping 554</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
         <v>21.75</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B17" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B18" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -3309,9 +3559,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3323,7 +3573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3470,6 +3720,22 @@
         <v>18.86</v>
       </c>
       <c r="D9" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>18.86</v>
+      </c>
+      <c r="D10" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -3488,7 +3754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3499,6 +3765,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3547,6 +3814,11 @@
       <c r="H2" s="24" t="inlineStr">
         <is>
           <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3565,6 +3837,7 @@
       <c r="F3" s="19" t="n"/>
       <c r="G3" s="19" t="n"/>
       <c r="H3" s="19" t="n"/>
+      <c r="I3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3591,6 +3864,9 @@
         <v>11.5</v>
       </c>
       <c r="H4" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="I4" s="21" t="n">
         <v>11.5</v>
       </c>
     </row>
@@ -3619,6 +3895,7 @@
       <c r="H5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="I5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3645,10 +3922,13 @@
       <c r="H6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="I6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3661,7 +3941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3672,6 +3952,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3722,6 +4003,11 @@
           <t>2026-05-31</t>
         </is>
       </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3750,6 +4036,9 @@
       <c r="H3" s="19" t="n">
         <v>21.75</v>
       </c>
+      <c r="I3" s="19" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3776,6 +4065,9 @@
         <v>16.84</v>
       </c>
       <c r="H4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="I4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -3804,6 +4096,7 @@
       <c r="H5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="I5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -3832,10 +4125,13 @@
       <c r="H6" s="21" t="n">
         <v>17.99</v>
       </c>
+      <c r="I6" s="21" t="n">
+        <v>17.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3848,7 +4144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3859,6 +4155,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3909,6 +4206,11 @@
           <t>2026-05-31</t>
         </is>
       </c>
+      <c r="I2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3937,6 +4239,9 @@
       <c r="H3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="I3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -3965,10 +4270,13 @@
       <c r="H4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="I4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3981,7 +4289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7150,6 +7458,681 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B128" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C128" s="33" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D128" s="21" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E128" s="33" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B129" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C129" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D129" s="19" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E129" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B130" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C130" s="33" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D130" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E130" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B131" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C131" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D131" s="19" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E131" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B132" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C132" s="33" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D132" s="21" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E132" s="33" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B133" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C133" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D133" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E133" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B134" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C134" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D134" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E134" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B135" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C135" s="32" t="inlineStr">
+        <is>
+          <t>ModregoHogar BP795</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="n">
+        <v>394</v>
+      </c>
+      <c r="E135" s="32" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/espumas-de-poliuretano/masilla-poliuretano-bostik-seal-n-flex-p795-gris-290ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B136" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C136" s="33" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D136" s="21" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E136" s="33" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B137" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C137" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D137" s="19" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E137" s="32" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B138" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C138" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D138" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E138" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B139" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C139" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D139" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E139" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B140" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C140" s="33" t="inlineStr">
+        <is>
+          <t>SVB Marine 591</t>
+        </is>
+      </c>
+      <c r="D140" s="21" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="E140" s="33" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sellador-marino-sikaflex-591.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B141" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C141" s="32" t="inlineStr">
+        <is>
+          <t>Francobordo 591</t>
+        </is>
+      </c>
+      <c r="D141" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E141" s="32" t="inlineStr">
+        <is>
+          <t>https://www.francobordo.com/sikaflex-591-sellador-de-bajas-emisiones-p-352421.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B142" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C142" s="33" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D142" s="21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E142" s="33" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B143" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C143" s="32" t="inlineStr">
+        <is>
+          <t>SVB Marine 291i</t>
+        </is>
+      </c>
+      <c r="D143" s="19" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="E143" s="32" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sikaflex-sellador-marino-291i-para-juntas.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B144" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C144" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D144" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E144" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B145" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C145" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D145" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E145" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B146" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C146" s="33" t="inlineStr">
+        <is>
+          <t>Francobordo 3M5200</t>
+        </is>
+      </c>
+      <c r="D146" s="21" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E146" s="33" t="inlineStr">
+        <is>
+          <t>https://www.francobordo.com/3m-adhesivo-sellador-marine-5200-blanco-p-353215.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B147" s="32" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C147" s="32" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D147" s="19" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E147" s="32" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B148" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C148" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D148" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E148" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B149" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C149" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D149" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E149" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B150" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C150" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D150" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E150" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B151" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C151" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D151" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E151" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B152" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C152" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D152" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E152" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B153" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C153" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D153" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E153" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B154" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C154" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D154" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E154" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-02
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$10</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$10</f>
+              <f>'📊 Media diaria'!$A$3:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$11</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$10</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$10</f>
+              <f>'📊 Media diaria'!$A$3:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$11</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$10</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$10</f>
+              <f>'📊 Media diaria'!$A$3:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -731,6 +731,33 @@
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -749,39 +776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$3</f>
             </numRef>
           </val>
         </ser>
@@ -803,12 +803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -830,12 +830,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -857,12 +857,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -884,12 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -911,12 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -938,18 +938,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -968,66 +1022,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="17"/>
-          <order val="17"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1049,12 +1049,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1076,12 +1076,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1103,12 +1103,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1130,12 +1130,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1157,18 +1157,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1187,93 +1268,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="24"/>
-          <order val="24"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="25"/>
-          <order val="25"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="26"/>
-          <order val="26"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -1295,12 +1295,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1322,12 +1322,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1349,12 +1349,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1376,18 +1376,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="31"/>
           <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1406,12 +1514,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -1520,7 +1628,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1547,7 +1655,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1574,7 +1682,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1601,7 +1709,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1628,7 +1736,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1655,7 +1763,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1682,7 +1790,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -1694,6 +1802,33 @@
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1712,39 +1847,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$3</f>
             </numRef>
           </val>
         </ser>
@@ -1766,12 +1874,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1793,12 +1901,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1820,12 +1928,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1847,12 +1955,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1874,12 +1982,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1901,18 +2009,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -1931,66 +2093,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="17"/>
-          <order val="17"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -2012,12 +2120,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2039,12 +2147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2066,12 +2174,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2093,12 +2201,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2120,18 +2228,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -2150,93 +2339,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="24"/>
-          <order val="24"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="25"/>
-          <order val="25"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="26"/>
-          <order val="26"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -2258,12 +2366,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -2285,12 +2393,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -2312,12 +2420,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2339,18 +2447,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="31"/>
           <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -2369,120 +2585,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="32"/>
-          <order val="32"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="33"/>
-          <order val="33"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="34"/>
-          <order val="34"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="35"/>
-          <order val="35"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -2504,12 +2612,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -2531,12 +2639,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -2558,18 +2666,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="39"/>
           <order val="39"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="41"/>
+          <order val="41"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="42"/>
+          <order val="42"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="43"/>
+          <order val="43"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="44"/>
+          <order val="44"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -2588,12 +2831,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
             </numRef>
           </val>
         </ser>
@@ -2702,7 +2945,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2729,7 +2972,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2756,7 +2999,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2783,7 +3026,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2810,7 +3053,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2837,7 +3080,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2864,7 +3107,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
             </numRef>
           </cat>
           <val>
@@ -2876,6 +3119,33 @@
         <ser>
           <idx val="7"/>
           <order val="7"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -2894,39 +3164,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$3</f>
             </numRef>
           </val>
         </ser>
@@ -2948,12 +3191,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2975,12 +3218,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -3002,12 +3245,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -3029,12 +3272,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -3056,12 +3299,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -3083,18 +3326,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -3113,12 +3410,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$I$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -3193,7 +3490,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -3604,14 +3901,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 01/06/2026 21:08</t>
+          <t>Última actualización: 02/06/2026 19:05</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-01</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3970,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-01</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -3710,21 +4007,21 @@
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>TodoCampers 554</t>
+          <t>Intercut 554</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>13.93</v>
+        <v>16.84</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
+          <t>TodoCampers 554</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>16.84</v>
+        <v>16.85</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -3745,7 +4042,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-01</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -3812,7 +4109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3975,6 +4272,22 @@
         <v>14.44</v>
       </c>
       <c r="D10" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="D11" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -3993,7 +4306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4005,6 +4318,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4058,6 +4372,11 @@
       <c r="I2" s="24" t="inlineStr">
         <is>
           <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="J2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -4079,6 +4398,9 @@
       <c r="I3" s="19" t="n">
         <v>5.97</v>
       </c>
+      <c r="J3" s="19" t="n">
+        <v>5.97</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4108,6 +4430,9 @@
         <v>11.5</v>
       </c>
       <c r="I4" s="21" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="J4" s="21" t="n">
         <v>9.1</v>
       </c>
     </row>
@@ -4137,6 +4462,7 @@
         <v>12.4</v>
       </c>
       <c r="I5" s="19" t="n"/>
+      <c r="J5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -4166,10 +4492,13 @@
       <c r="I6" s="21" t="n">
         <v>9.9</v>
       </c>
+      <c r="J6" s="21" t="n">
+        <v>9.9</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4182,7 +4511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4194,6 +4523,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4249,6 +4579,11 @@
           <t>2026-06-01</t>
         </is>
       </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4280,6 +4615,9 @@
       <c r="I3" s="19" t="n">
         <v>8.99</v>
       </c>
+      <c r="J3" s="19" t="n">
+        <v>8.99</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4309,6 +4647,9 @@
         <v>16.84</v>
       </c>
       <c r="I4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="J4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -4338,6 +4679,7 @@
         <v>18.87</v>
       </c>
       <c r="I5" s="19" t="n"/>
+      <c r="J5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -4367,6 +4709,9 @@
         <v>17.99</v>
       </c>
       <c r="I6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="J6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -4386,10 +4731,13 @@
       <c r="I7" s="19" t="n">
         <v>13.93</v>
       </c>
+      <c r="J7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4402,7 +4750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4414,6 +4762,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4469,6 +4818,11 @@
           <t>2026-06-01</t>
         </is>
       </c>
+      <c r="J2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4500,6 +4854,9 @@
       <c r="I3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="J3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4531,10 +4888,13 @@
       <c r="I4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="J4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4547,7 +4907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8491,6 +8851,681 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B159" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C159" s="32" t="inlineStr">
+        <is>
+          <t>Andorra Campers</t>
+        </is>
+      </c>
+      <c r="D159" s="19" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="E159" s="32" t="inlineStr">
+        <is>
+          <t>https://www.andorracampers.com/es/sikaflex-522-blanca_3485_342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B160" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C160" s="33" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D160" s="21" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E160" s="33" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B161" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C161" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D161" s="19" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E161" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B162" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C162" s="33" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D162" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E162" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B163" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C163" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D163" s="19" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E163" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B164" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C164" s="33" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D164" s="21" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E164" s="33" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B165" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C165" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D165" s="19" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="E165" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B166" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C166" s="33" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D166" s="21" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E166" s="33" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B167" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C167" s="32" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D167" s="19" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E167" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B168" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C168" s="33" t="inlineStr">
+        <is>
+          <t>ModregoHogar BP795</t>
+        </is>
+      </c>
+      <c r="D168" s="21" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E168" s="33" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/espumas-de-poliuretano/masilla-poliuretano-bostik-seal-n-flex-p795-gris-290ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B169" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C169" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D169" s="19" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="E169" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B170" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C170" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D170" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E170" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B171" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C171" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D171" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E171" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B172" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C172" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D172" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E172" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B173" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C173" s="32" t="inlineStr">
+        <is>
+          <t>SVB Marine 591</t>
+        </is>
+      </c>
+      <c r="D173" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E173" s="32" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sellador-marino-sikaflex-591.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B174" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C174" s="33" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D174" s="21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E174" s="33" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B175" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C175" s="32" t="inlineStr">
+        <is>
+          <t>SVB Marine 291i</t>
+        </is>
+      </c>
+      <c r="D175" s="19" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="E175" s="32" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sikaflex-sellador-marino-291i-para-juntas.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B176" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C176" s="33" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D176" s="21" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E176" s="33" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B177" s="32" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C177" s="32" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D177" s="19" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E177" s="32" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B178" s="33" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C178" s="33" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D178" s="21" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="E178" s="33" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B179" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C179" s="32" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D179" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E179" s="32" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B180" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C180" s="33" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D180" s="21" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E180" s="33" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B181" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C181" s="32" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D181" s="19" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E181" s="32" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B182" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C182" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D182" s="21" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E182" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B183" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C183" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D183" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E183" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B184" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C184" s="33" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D184" s="21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E184" s="33" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B185" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C185" s="32" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D185" s="19" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E185" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-03
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$11</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$11</f>
+              <f>'📊 Media diaria'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$12</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$11</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$11</f>
+              <f>'📊 Media diaria'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$12</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$11</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$11</f>
+              <f>'📊 Media diaria'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -758,6 +758,33 @@
         <ser>
           <idx val="8"/>
           <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -776,39 +803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="9"/>
-          <order val="9"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$3</f>
             </numRef>
           </val>
         </ser>
@@ -830,12 +830,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -857,12 +857,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -884,12 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -911,12 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -938,12 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,18 +992,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1022,66 +1076,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -1103,12 +1103,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1130,12 +1130,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1157,12 +1157,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1184,12 +1184,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1211,12 +1211,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1238,18 +1238,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="26"/>
           <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1268,93 +1349,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="27"/>
-          <order val="27"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="28"/>
-          <order val="28"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="29"/>
-          <order val="29"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -1376,12 +1376,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1403,12 +1403,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1430,12 +1430,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1457,12 +1457,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1484,18 +1484,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="35"/>
           <order val="35"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="36"/>
+          <order val="36"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="37"/>
+          <order val="37"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="38"/>
+          <order val="38"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="39"/>
+          <order val="39"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1514,12 +1622,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -1628,7 +1736,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1655,7 +1763,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1682,7 +1790,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1709,7 +1817,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1736,7 +1844,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1763,7 +1871,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1790,7 +1898,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1817,7 +1925,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -1829,6 +1937,33 @@
         <ser>
           <idx val="8"/>
           <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1847,39 +1982,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="9"/>
-          <order val="9"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$3</f>
             </numRef>
           </val>
         </ser>
@@ -1901,12 +2009,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1928,12 +2036,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1955,12 +2063,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1982,12 +2090,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2009,12 +2117,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2036,12 +2144,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2063,18 +2171,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2093,66 +2255,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -2174,12 +2282,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2201,12 +2309,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2228,12 +2336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2255,12 +2363,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2282,12 +2390,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2309,18 +2417,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="26"/>
           <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -2339,93 +2528,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="27"/>
-          <order val="27"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="28"/>
-          <order val="28"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="29"/>
-          <order val="29"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -2447,12 +2555,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2582,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -2501,12 +2609,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2528,12 +2636,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2555,18 +2663,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="35"/>
           <order val="35"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="36"/>
+          <order val="36"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="37"/>
+          <order val="37"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="38"/>
+          <order val="38"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="39"/>
+          <order val="39"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -2585,120 +2801,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="36"/>
-          <order val="36"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="37"/>
-          <order val="37"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="38"/>
-          <order val="38"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="39"/>
-          <order val="39"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -2720,12 +2828,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -2747,12 +2855,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -2774,12 +2882,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -2801,18 +2909,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="44"/>
           <order val="44"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="45"/>
+          <order val="45"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="46"/>
+          <order val="46"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="47"/>
+          <order val="47"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="48"/>
+          <order val="48"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="49"/>
+          <order val="49"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -2831,12 +3074,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
             </numRef>
           </val>
         </ser>
@@ -2945,7 +3188,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -2972,7 +3215,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -2999,7 +3242,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3026,7 +3269,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3053,7 +3296,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3080,7 +3323,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3107,7 +3350,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3134,7 +3377,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
             </numRef>
           </cat>
           <val>
@@ -3146,6 +3389,33 @@
         <ser>
           <idx val="8"/>
           <order val="8"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -3164,39 +3434,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="9"/>
-          <order val="9"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$3</f>
             </numRef>
           </val>
         </ser>
@@ -3218,12 +3461,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -3245,12 +3488,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -3272,12 +3515,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -3299,12 +3542,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -3326,12 +3569,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -3353,12 +3596,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -3380,18 +3623,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="17"/>
           <order val="17"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -3410,12 +3707,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$J$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -3490,7 +3787,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -3881,7 +4178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3901,14 +4198,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 02/06/2026 19:05</t>
+          <t>Última actualización: 03/06/2026 20:04</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-02</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -3958,134 +4255,154 @@
           <t>Obelink 522</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>9.9</v>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Berger Camping 554</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
-      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>16.84</v>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>TodoCampers 554</t>
+          <t>Intercut 554</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>16.85</v>
+        <v>16.84</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>16.85</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>Obelink 554</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B16" s="8" t="n">
         <v>17.99</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B21" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B22" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -4095,9 +4412,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4109,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4288,6 +4605,22 @@
         <v>15.17</v>
       </c>
       <c r="D11" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>15.91</v>
+      </c>
+      <c r="D12" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -4306,7 +4639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4319,6 +4652,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4377,6 +4711,11 @@
       <c r="J2" s="24" t="inlineStr">
         <is>
           <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="K2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -4401,6 +4740,9 @@
       <c r="J3" s="19" t="n">
         <v>5.97</v>
       </c>
+      <c r="K3" s="19" t="n">
+        <v>5.97</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4433,6 +4775,9 @@
         <v>9.1</v>
       </c>
       <c r="J4" s="21" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K4" s="21" t="n">
         <v>9.1</v>
       </c>
     </row>
@@ -4463,6 +4808,9 @@
       </c>
       <c r="I5" s="19" t="n"/>
       <c r="J5" s="19" t="n"/>
+      <c r="K5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -4495,10 +4843,13 @@
       <c r="J6" s="21" t="n">
         <v>9.9</v>
       </c>
+      <c r="K6" s="21" t="n">
+        <v>9.9</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4511,7 +4862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4524,6 +4875,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4584,6 +4936,11 @@
           <t>2026-06-02</t>
         </is>
       </c>
+      <c r="K2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4618,6 +4975,9 @@
       <c r="J3" s="19" t="n">
         <v>8.99</v>
       </c>
+      <c r="K3" s="19" t="n">
+        <v>8.99</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4650,6 +5010,9 @@
         <v>16.84</v>
       </c>
       <c r="J4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="K4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -4680,6 +5043,9 @@
       </c>
       <c r="I5" s="19" t="n"/>
       <c r="J5" s="19" t="n"/>
+      <c r="K5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -4712,6 +5078,9 @@
         <v>17.99</v>
       </c>
       <c r="J6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="K6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -4734,10 +5103,13 @@
       <c r="J7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="K7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4750,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4763,6 +5135,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4823,6 +5196,11 @@
           <t>2026-06-02</t>
         </is>
       </c>
+      <c r="K2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4857,6 +5235,9 @@
       <c r="J3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="K3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4891,10 +5272,13 @@
       <c r="J4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="K4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4907,7 +5291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:F216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9526,6 +9910,781 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B186" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C186" s="33" t="inlineStr">
+        <is>
+          <t>Andorra Campers</t>
+        </is>
+      </c>
+      <c r="D186" s="21" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="E186" s="33" t="inlineStr">
+        <is>
+          <t>https://www.andorracampers.com/es/sikaflex-522-blanca_3485_342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B187" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C187" s="32" t="inlineStr">
+        <is>
+          <t>Barna Campers</t>
+        </is>
+      </c>
+      <c r="D187" s="19" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E187" s="32" t="inlineStr">
+        <is>
+          <t>https://barnacampers.es/Sikaflex-52-BLANCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B188" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C188" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D188" s="21" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E188" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B189" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C189" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D189" s="19" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E189" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B190" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C190" s="33" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D190" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E190" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B191" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C191" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D191" s="19" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E191" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B192" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C192" s="33" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D192" s="21" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E192" s="33" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B193" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C193" s="32" t="inlineStr">
+        <is>
+          <t>Berger Camping 554</t>
+        </is>
+      </c>
+      <c r="D193" s="19" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="E193" s="32" t="inlineStr">
+        <is>
+          <t>https://www.berger-camping.es/producto/adhesivo-de-montaje-sikaflex-554-sika-217196</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B194" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C194" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D194" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E194" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B195" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C195" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D195" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E195" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B196" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C196" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D196" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E196" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B197" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C197" s="32" t="inlineStr">
+        <is>
+          <t>ModregoHogar BP795</t>
+        </is>
+      </c>
+      <c r="D197" s="19" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E197" s="32" t="inlineStr">
+        <is>
+          <t>https://www.modregohogar.com/ferreteria/silicona/espumas-de-poliuretano/masilla-poliuretano-bostik-seal-n-flex-p795-gris-290ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B198" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C198" s="33" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D198" s="21" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="E198" s="33" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B199" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C199" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D199" s="19" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E199" s="32" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B200" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C200" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D200" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E200" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B201" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C201" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D201" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E201" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B202" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C202" s="33" t="inlineStr">
+        <is>
+          <t>SVB Marine 591</t>
+        </is>
+      </c>
+      <c r="D202" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E202" s="33" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sellador-marino-sikaflex-591.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B203" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C203" s="32" t="inlineStr">
+        <is>
+          <t>Francobordo 591</t>
+        </is>
+      </c>
+      <c r="D203" s="19" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E203" s="32" t="inlineStr">
+        <is>
+          <t>https://www.francobordo.com/sikaflex-591-sellador-de-bajas-emisiones-p-352421.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B204" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C204" s="33" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D204" s="21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E204" s="33" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B205" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C205" s="32" t="inlineStr">
+        <is>
+          <t>SVB Marine 291i</t>
+        </is>
+      </c>
+      <c r="D205" s="19" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E205" s="32" t="inlineStr">
+        <is>
+          <t>https://www.svb-marine.es/es/sika-sikaflex-sellador-marino-291i-para-juntas.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B206" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C206" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D206" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E206" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B207" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C207" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D207" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E207" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B208" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C208" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D208" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E208" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B209" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C209" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D209" s="19" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="E209" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B210" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C210" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D210" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E210" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B211" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C211" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D211" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E211" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B212" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C212" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D212" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E212" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B213" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C213" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D213" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E213" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B214" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C214" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D214" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E214" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B215" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C215" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D215" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E215" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B216" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C216" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D216" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E216" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-04
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -174,15 +174,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$12</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$12</f>
+              <f>'📊 Media diaria'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$12</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$12</f>
+              <f>'📊 Media diaria'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$13</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$12</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$12</f>
+              <f>'📊 Media diaria'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -785,6 +785,33 @@
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -803,39 +830,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="10"/>
-          <order val="10"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$3</f>
             </numRef>
           </val>
         </ser>
@@ -857,12 +857,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -884,12 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -911,12 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -938,12 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,18 +1046,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="19"/>
           <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1076,66 +1130,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="21"/>
-          <order val="21"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -1157,12 +1157,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1184,12 +1184,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1211,12 +1211,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1238,12 +1238,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1265,12 +1265,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1292,12 +1292,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1319,18 +1319,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="29"/>
           <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1349,93 +1430,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="30"/>
-          <order val="30"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="31"/>
-          <order val="31"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="32"/>
-          <order val="32"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -1457,12 +1457,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1484,12 +1484,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1511,12 +1511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1538,12 +1538,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1565,12 +1565,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1592,18 +1592,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="39"/>
           <order val="39"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="41"/>
+          <order val="41"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="42"/>
+          <order val="42"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="43"/>
+          <order val="43"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1622,12 +1730,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
             </numRef>
           </val>
         </ser>
@@ -1736,7 +1844,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1763,7 +1871,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1790,7 +1898,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1817,7 +1925,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1844,7 +1952,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1871,7 +1979,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1898,7 +2006,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1925,7 +2033,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1952,7 +2060,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -1964,6 +2072,33 @@
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -1982,39 +2117,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="10"/>
-          <order val="10"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$3</f>
             </numRef>
           </val>
         </ser>
@@ -2036,12 +2144,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2063,12 +2171,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2090,12 +2198,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2117,12 +2225,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2144,12 +2252,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2171,12 +2279,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2198,12 +2306,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2225,18 +2333,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="19"/>
           <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2255,66 +2417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="21"/>
-          <order val="21"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -2336,12 +2444,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2363,12 +2471,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2390,12 +2498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2417,12 +2525,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2444,12 +2552,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2471,12 +2579,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -2498,18 +2606,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="29"/>
           <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -2528,93 +2717,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="30"/>
-          <order val="30"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="31"/>
-          <order val="31"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="32"/>
-          <order val="32"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -2636,12 +2744,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -2663,12 +2771,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -2690,12 +2798,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2717,12 +2825,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2744,12 +2852,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -2771,18 +2879,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="39"/>
           <order val="39"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="41"/>
+          <order val="41"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="42"/>
+          <order val="42"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="43"/>
+          <order val="43"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -2801,120 +3017,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="40"/>
-          <order val="40"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="41"/>
-          <order val="41"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="42"/>
-          <order val="42"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="43"/>
-          <order val="43"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
             </numRef>
           </val>
         </ser>
@@ -2936,12 +3044,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -2963,12 +3071,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -2990,12 +3098,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -3017,12 +3125,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -3044,18 +3152,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="49"/>
           <order val="49"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="50"/>
+          <order val="50"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="51"/>
+          <order val="51"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="52"/>
+          <order val="52"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="53"/>
+          <order val="53"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="54"/>
+          <order val="54"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -3074,12 +3317,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
             </numRef>
           </val>
         </ser>
@@ -3188,7 +3431,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3215,7 +3458,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3242,7 +3485,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3269,7 +3512,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3296,7 +3539,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3323,7 +3566,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3350,7 +3593,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3377,7 +3620,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3404,7 +3647,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
             </numRef>
           </cat>
           <val>
@@ -3416,6 +3659,33 @@
         <ser>
           <idx val="9"/>
           <order val="9"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -3434,39 +3704,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="10"/>
-          <order val="10"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$3</f>
             </numRef>
           </val>
         </ser>
@@ -3488,12 +3731,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -3515,12 +3758,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -3542,12 +3785,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -3569,12 +3812,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -3596,12 +3839,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -3623,12 +3866,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -3650,12 +3893,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -3677,18 +3920,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="19"/>
           <order val="19"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -3707,12 +4004,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$K$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -3787,7 +4084,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -4178,7 +4475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4198,14 +4495,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 03/06/2026 20:04</t>
+          <t>Última actualización: 04/06/2026 08:10</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-03</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -4227,11 +4524,11 @@
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Andorra Campers</t>
+          <t>Obelink 522</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>5.97</v>
+        <v>10.99</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
@@ -4242,167 +4539,137 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Barna Campers</t>
+          <t>Madrid Camper 522</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>9.1</v>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Obelink 522</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>9.9</v>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 522</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
         <v>12.4</v>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>16.85</v>
+      </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Berger Camping 554</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>17.99</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
+          <t>Madrid Camper 554</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>16.84</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>TodoCampers 554</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>16.85</v>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Obelink 554</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>17.99</v>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 554</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="n">
         <v>18.87</v>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n">
+      <c r="B18" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B19" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -4412,9 +4679,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4426,7 +4693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4621,6 +4888,22 @@
         <v>15.91</v>
       </c>
       <c r="D12" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D13" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -4639,7 +4922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4653,6 +4936,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4716,6 +5000,11 @@
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="L2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -4743,6 +5032,7 @@
       <c r="K3" s="19" t="n">
         <v>5.97</v>
       </c>
+      <c r="L3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -4780,6 +5070,7 @@
       <c r="K4" s="21" t="n">
         <v>9.1</v>
       </c>
+      <c r="L4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -4811,6 +5102,9 @@
       <c r="K5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="L5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -4846,10 +5140,13 @@
       <c r="K6" s="21" t="n">
         <v>9.9</v>
       </c>
+      <c r="L6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4862,7 +5159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4876,6 +5173,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4941,6 +5239,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="L2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4978,6 +5281,7 @@
       <c r="K3" s="19" t="n">
         <v>8.99</v>
       </c>
+      <c r="L3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5013,6 +5317,9 @@
         <v>16.84</v>
       </c>
       <c r="K4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="L4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -5046,6 +5353,9 @@
       <c r="K5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="L5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5081,6 +5391,9 @@
         <v>17.99</v>
       </c>
       <c r="K6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="L6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -5106,10 +5419,13 @@
       <c r="K7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="L7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5122,7 +5438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5136,6 +5452,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5201,6 +5518,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="L2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5238,6 +5560,9 @@
       <c r="K3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="L3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5275,10 +5600,13 @@
       <c r="K4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="L4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5291,7 +5619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F216"/>
+  <dimension ref="A1:F240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10685,6 +11013,606 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B217" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C217" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D217" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E217" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B218" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C218" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D218" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E218" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B219" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C219" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D219" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E219" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B220" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C220" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D220" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E220" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B221" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C221" s="32" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D221" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E221" s="32" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B222" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C222" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D222" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E222" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B223" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C223" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D223" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E223" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B224" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C224" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D224" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E224" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B225" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C225" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D225" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E225" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B226" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C226" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D226" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E226" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B227" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C227" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D227" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E227" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B228" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C228" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D228" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E228" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B229" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C229" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D229" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E229" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B230" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C230" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D230" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E230" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B231" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C231" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D231" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E231" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B232" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C232" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D232" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E232" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B233" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C233" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D233" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E233" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B234" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C234" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D234" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E234" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B235" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C235" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D235" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E235" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B236" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C236" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D236" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E236" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B237" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C237" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D237" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E237" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B238" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C238" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D238" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E238" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B239" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C239" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D239" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E239" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B240" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C240" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D240" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E240" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-05
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$13</f>
+              <f>'📊 Media diaria'!$A$3:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$13</f>
+              <f>'📊 Media diaria'!$A$3:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$13</f>
+              <f>'📊 Media diaria'!$A$3:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -812,6 +812,33 @@
         <ser>
           <idx val="10"/>
           <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -830,39 +857,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="11"/>
-          <order val="11"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$3</f>
             </numRef>
           </val>
         </ser>
@@ -884,12 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -911,12 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -938,12 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,18 +1100,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="21"/>
           <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1130,66 +1184,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="22"/>
-          <order val="22"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="23"/>
-          <order val="23"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -1211,12 +1211,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1238,12 +1238,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1265,12 +1265,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1292,12 +1292,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1319,12 +1319,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1346,12 +1346,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1373,12 +1373,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1400,18 +1400,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="32"/>
           <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1430,93 +1511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="33"/>
-          <order val="33"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="34"/>
-          <order val="34"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="35"/>
-          <order val="35"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
             </numRef>
           </val>
         </ser>
@@ -1538,12 +1538,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1565,12 +1565,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1592,12 +1592,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1619,12 +1619,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1646,12 +1646,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1673,12 +1673,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1700,18 +1700,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="43"/>
           <order val="43"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="44"/>
+          <order val="44"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="45"/>
+          <order val="45"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="46"/>
+          <order val="46"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="47"/>
+          <order val="47"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1730,12 +1838,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
             </numRef>
           </val>
         </ser>
@@ -1844,7 +1952,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -1871,7 +1979,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -1898,7 +2006,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -1925,7 +2033,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -1952,7 +2060,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -1979,7 +2087,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -2006,7 +2114,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -2033,7 +2141,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -2060,7 +2168,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -2087,7 +2195,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -2099,6 +2207,33 @@
         <ser>
           <idx val="10"/>
           <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2117,39 +2252,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="11"/>
-          <order val="11"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$3</f>
             </numRef>
           </val>
         </ser>
@@ -2171,12 +2279,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2198,12 +2306,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2225,12 +2333,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2252,12 +2360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2279,12 +2387,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2306,12 +2414,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2333,12 +2441,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2360,12 +2468,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2387,18 +2495,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="21"/>
           <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2417,66 +2579,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="22"/>
-          <order val="22"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="23"/>
-          <order val="23"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -2498,12 +2606,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2525,12 +2633,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2552,12 +2660,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2579,12 +2687,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2606,12 +2714,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2633,12 +2741,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -2660,12 +2768,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2687,18 +2795,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="32"/>
           <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -2717,93 +2906,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="33"/>
-          <order val="33"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="34"/>
-          <order val="34"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="35"/>
-          <order val="35"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
             </numRef>
           </val>
         </ser>
@@ -2825,12 +2933,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -2852,12 +2960,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -2879,12 +2987,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2906,12 +3014,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2933,12 +3041,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -2960,12 +3068,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -2987,18 +3095,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="43"/>
           <order val="43"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="44"/>
+          <order val="44"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="45"/>
+          <order val="45"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="46"/>
+          <order val="46"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="47"/>
+          <order val="47"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -3017,120 +3233,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="44"/>
-          <order val="44"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="45"/>
-          <order val="45"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="46"/>
-          <order val="46"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="47"/>
-          <order val="47"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
             </numRef>
           </val>
         </ser>
@@ -3152,12 +3260,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -3179,12 +3287,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -3206,12 +3314,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -3233,12 +3341,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -3260,12 +3368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -3287,18 +3395,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="54"/>
           <order val="54"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="55"/>
+          <order val="55"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="56"/>
+          <order val="56"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="57"/>
+          <order val="57"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="58"/>
+          <order val="58"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="59"/>
+          <order val="59"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -3317,12 +3560,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
             </numRef>
           </val>
         </ser>
@@ -3431,7 +3674,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3458,7 +3701,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3485,7 +3728,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3512,7 +3755,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3539,7 +3782,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3566,7 +3809,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3593,7 +3836,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3620,7 +3863,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3647,7 +3890,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3674,7 +3917,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
             </numRef>
           </cat>
           <val>
@@ -3686,6 +3929,33 @@
         <ser>
           <idx val="10"/>
           <order val="10"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -3704,39 +3974,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="11"/>
-          <order val="11"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$3</f>
             </numRef>
           </val>
         </ser>
@@ -3758,12 +4001,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -3785,12 +4028,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -3812,12 +4055,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -3839,12 +4082,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -3866,12 +4109,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -3893,12 +4136,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -3920,12 +4163,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -3947,12 +4190,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -3974,18 +4217,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="21"/>
           <order val="21"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -4004,12 +4301,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$L$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -4084,7 +4381,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -4495,14 +4792,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 04/06/2026 17:37</t>
+          <t>Última actualización: 05/06/2026 16:19</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-04</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4851,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-04</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4923,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-04</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4904,6 +5201,22 @@
         <v>17.64</v>
       </c>
       <c r="D13" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D14" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -4922,7 +5235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4937,6 +5250,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5005,6 +5319,11 @@
       <c r="L2" s="24" t="inlineStr">
         <is>
           <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="M2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -5033,6 +5352,7 @@
         <v>5.97</v>
       </c>
       <c r="L3" s="19" t="n"/>
+      <c r="M3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5071,6 +5391,7 @@
         <v>9.1</v>
       </c>
       <c r="L4" s="21" t="n"/>
+      <c r="M4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -5105,6 +5426,9 @@
       <c r="L5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="M5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5143,10 +5467,13 @@
       <c r="L6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="M6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5159,7 +5486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5174,6 +5501,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5244,6 +5572,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="M2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5282,6 +5615,7 @@
         <v>8.99</v>
       </c>
       <c r="L3" s="19" t="n"/>
+      <c r="M3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5320,6 +5654,9 @@
         <v>16.84</v>
       </c>
       <c r="L4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="M4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -5356,6 +5693,9 @@
       <c r="L5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="M5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5394,6 +5734,9 @@
         <v>17.99</v>
       </c>
       <c r="L6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="M6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -5422,10 +5765,13 @@
       <c r="L7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="M7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5438,7 +5784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5453,6 +5799,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5523,6 +5870,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="M2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5563,6 +5915,9 @@
       <c r="L3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="M3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5603,10 +5958,13 @@
       <c r="L4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="M4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5619,7 +5977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F240"/>
+  <dimension ref="A1:F264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11613,6 +11971,606 @@
         </is>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B241" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C241" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D241" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E241" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B242" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C242" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D242" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E242" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B243" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C243" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D243" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E243" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B244" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C244" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D244" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E244" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B245" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C245" s="32" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D245" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E245" s="32" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B246" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C246" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D246" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E246" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B247" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C247" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D247" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E247" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B248" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C248" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D248" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E248" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B249" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C249" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D249" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E249" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B250" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C250" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D250" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E250" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B251" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C251" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D251" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E251" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B252" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C252" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D252" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E252" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B253" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C253" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D253" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E253" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B254" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C254" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D254" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E254" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B255" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C255" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D255" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E255" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B256" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C256" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D256" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E256" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B257" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C257" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D257" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E257" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B258" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C258" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D258" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E258" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B259" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C259" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D259" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E259" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B260" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C260" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D260" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E260" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B261" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C261" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D261" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E261" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B262" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C262" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D262" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E262" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B263" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C263" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D263" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E263" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B264" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C264" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D264" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E264" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-06
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$14</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$14</f>
+              <f>'📊 Media diaria'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$15</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$14</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$14</f>
+              <f>'📊 Media diaria'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$15</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$14</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$14</f>
+              <f>'📊 Media diaria'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$15</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -827,7 +827,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -839,6 +839,33 @@
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -857,39 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$3</f>
             </numRef>
           </val>
         </ser>
@@ -911,12 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -938,12 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1127,12 +1127,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1154,18 +1154,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1184,66 +1238,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="24"/>
-          <order val="24"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="25"/>
-          <order val="25"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -1265,12 +1265,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1292,12 +1292,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1319,12 +1319,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1346,12 +1346,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1373,12 +1373,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1400,12 +1400,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1427,12 +1427,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1454,12 +1454,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1481,18 +1481,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="35"/>
           <order val="35"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="36"/>
+          <order val="36"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="37"/>
+          <order val="37"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="38"/>
+          <order val="38"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1511,93 +1592,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="36"/>
-          <order val="36"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="37"/>
-          <order val="37"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="38"/>
-          <order val="38"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$5</f>
             </numRef>
           </val>
         </ser>
@@ -1619,12 +1619,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1646,12 +1646,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1673,12 +1673,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1700,12 +1700,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1727,12 +1727,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1754,12 +1754,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1781,12 +1781,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1808,18 +1808,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="47"/>
           <order val="47"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="48"/>
+          <order val="48"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="49"/>
+          <order val="49"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="50"/>
+          <order val="50"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="51"/>
+          <order val="51"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1838,12 +1946,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$6</f>
             </numRef>
           </val>
         </ser>
@@ -1952,7 +2060,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -1979,7 +2087,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2006,7 +2114,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2033,7 +2141,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2060,7 +2168,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2087,7 +2195,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2114,7 +2222,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2141,7 +2249,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2168,7 +2276,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2195,7 +2303,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2222,7 +2330,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -2234,6 +2342,33 @@
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2252,39 +2387,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$3</f>
             </numRef>
           </val>
         </ser>
@@ -2306,12 +2414,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2333,12 +2441,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2360,12 +2468,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2387,12 +2495,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2414,12 +2522,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2441,12 +2549,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2468,12 +2576,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2495,12 +2603,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2522,12 +2630,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -2549,18 +2657,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2579,66 +2741,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="24"/>
-          <order val="24"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="25"/>
-          <order val="25"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -2660,12 +2768,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2687,12 +2795,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2714,12 +2822,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2741,12 +2849,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2768,12 +2876,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2795,12 +2903,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -2822,12 +2930,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2849,12 +2957,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -2876,18 +2984,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="35"/>
           <order val="35"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="36"/>
+          <order val="36"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="37"/>
+          <order val="37"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="38"/>
+          <order val="38"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -2906,93 +3095,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="36"/>
-          <order val="36"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="37"/>
-          <order val="37"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="38"/>
-          <order val="38"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$5</f>
             </numRef>
           </val>
         </ser>
@@ -3014,12 +3122,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -3041,12 +3149,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -3068,12 +3176,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -3095,12 +3203,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -3122,12 +3230,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -3149,12 +3257,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -3176,12 +3284,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3203,18 +3311,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="47"/>
           <order val="47"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="48"/>
+          <order val="48"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="49"/>
+          <order val="49"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="50"/>
+          <order val="50"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="51"/>
+          <order val="51"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -3233,120 +3449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="48"/>
-          <order val="48"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="49"/>
-          <order val="49"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="50"/>
-          <order val="50"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="51"/>
-          <order val="51"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$6</f>
             </numRef>
           </val>
         </ser>
@@ -3368,12 +3476,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -3395,12 +3503,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -3422,12 +3530,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -3449,12 +3557,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -3476,12 +3584,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -3503,12 +3611,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
@@ -3530,18 +3638,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="59"/>
           <order val="59"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="60"/>
+          <order val="60"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="61"/>
+          <order val="61"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="62"/>
+          <order val="62"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="63"/>
+          <order val="63"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="64"/>
+          <order val="64"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -3560,12 +3803,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$7</f>
             </numRef>
           </val>
         </ser>
@@ -3674,7 +3917,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3701,7 +3944,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3728,7 +3971,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3755,7 +3998,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3782,7 +4025,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3809,7 +4052,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3836,7 +4079,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3863,7 +4106,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3890,7 +4133,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3917,7 +4160,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3944,7 +4187,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
             </numRef>
           </cat>
           <val>
@@ -3956,6 +4199,33 @@
         <ser>
           <idx val="11"/>
           <order val="11"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -3974,39 +4244,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$3</f>
             </numRef>
           </val>
         </ser>
@@ -4028,12 +4271,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -4055,12 +4298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -4082,12 +4325,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -4109,12 +4352,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -4136,12 +4379,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -4163,12 +4406,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -4190,12 +4433,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -4217,12 +4460,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -4244,12 +4487,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -4271,18 +4514,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="23"/>
           <order val="23"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -4301,12 +4598,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$M$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -4381,7 +4678,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -4792,14 +5089,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 05/06/2026 16:19</t>
+          <t>Última actualización: 06/06/2026 11:16</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-05</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -4851,7 +5148,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-05</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -4923,7 +5220,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-05</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -4990,7 +5287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5217,6 +5514,22 @@
         <v>17.64</v>
       </c>
       <c r="D14" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D15" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -5235,7 +5548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5251,6 +5564,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5324,6 +5638,11 @@
       <c r="M2" s="24" t="inlineStr">
         <is>
           <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="N2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -5353,6 +5672,7 @@
       </c>
       <c r="L3" s="19" t="n"/>
       <c r="M3" s="19" t="n"/>
+      <c r="N3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5392,6 +5712,7 @@
       </c>
       <c r="L4" s="21" t="n"/>
       <c r="M4" s="21" t="n"/>
+      <c r="N4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -5429,6 +5750,9 @@
       <c r="M5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="N5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5470,10 +5794,13 @@
       <c r="M6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="N6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5486,7 +5813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5502,6 +5829,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5577,6 +5905,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="N2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5616,6 +5949,7 @@
       </c>
       <c r="L3" s="19" t="n"/>
       <c r="M3" s="19" t="n"/>
+      <c r="N3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5657,6 +5991,9 @@
         <v>16.84</v>
       </c>
       <c r="M4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="N4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -5696,6 +6033,9 @@
       <c r="M5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="N5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5737,6 +6077,9 @@
         <v>17.99</v>
       </c>
       <c r="M6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="N6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -5768,10 +6111,13 @@
       <c r="M7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="N7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5784,7 +6130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5800,6 +6146,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5875,6 +6222,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="N2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5918,6 +6270,9 @@
       <c r="M3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="N3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5961,10 +6316,13 @@
       <c r="M4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="N4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5977,7 +6335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F264"/>
+  <dimension ref="A1:F287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12571,6 +12929,581 @@
         </is>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B265" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C265" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D265" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E265" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B266" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C266" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D266" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E266" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B267" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C267" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D267" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E267" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B268" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C268" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D268" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E268" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B269" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C269" s="32" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D269" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E269" s="32" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B270" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C270" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D270" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E270" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B271" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C271" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D271" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E271" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B272" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C272" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D272" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E272" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B273" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C273" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D273" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E273" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B274" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C274" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D274" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E274" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B275" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C275" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D275" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E275" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B276" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C276" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D276" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E276" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B277" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C277" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D277" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E277" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B278" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C278" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D278" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E278" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B279" s="32" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C279" s="32" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D279" s="19" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E279" s="32" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B280" s="33" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C280" s="33" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D280" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E280" s="33" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B281" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C281" s="32" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D281" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E281" s="32" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B282" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C282" s="33" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D282" s="21" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E282" s="33" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B283" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C283" s="32" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D283" s="19" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E283" s="32" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B284" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C284" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D284" s="21" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E284" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B285" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C285" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D285" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E285" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B286" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C286" s="33" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D286" s="21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E286" s="33" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B287" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C287" s="32" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D287" s="19" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E287" s="32" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-07
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$15</f>
+              <f>'📊 Media diaria'!$A$3:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$15</f>
+              <f>'📊 Media diaria'!$A$3:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$16</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$15</f>
+              <f>'📊 Media diaria'!$A$3:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -827,7 +827,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -854,7 +854,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -866,6 +866,33 @@
         <ser>
           <idx val="12"/>
           <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -884,39 +911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$3</f>
             </numRef>
           </val>
         </ser>
@@ -938,12 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1127,12 +1127,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1154,12 +1154,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1181,12 +1181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -1208,18 +1208,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="25"/>
           <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1238,66 +1292,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="26"/>
-          <order val="26"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="27"/>
-          <order val="27"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$4</f>
             </numRef>
           </val>
         </ser>
@@ -1319,12 +1319,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1346,12 +1346,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1373,12 +1373,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1400,12 +1400,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1427,12 +1427,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1454,12 +1454,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1481,12 +1481,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1508,12 +1508,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1535,12 +1535,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -1562,18 +1562,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="38"/>
           <order val="38"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="39"/>
+          <order val="39"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="41"/>
+          <order val="41"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1592,93 +1673,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="39"/>
-          <order val="39"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="40"/>
-          <order val="40"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="41"/>
-          <order val="41"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$5</f>
             </numRef>
           </val>
         </ser>
@@ -1700,12 +1700,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1727,12 +1727,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1754,12 +1754,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1781,12 +1781,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1808,12 +1808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1835,12 +1835,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1862,12 +1862,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1889,12 +1889,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1916,18 +1916,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="51"/>
           <order val="51"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="52"/>
+          <order val="52"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="53"/>
+          <order val="53"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="54"/>
+          <order val="54"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="55"/>
+          <order val="55"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -1946,12 +2054,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$6</f>
             </numRef>
           </val>
         </ser>
@@ -2060,7 +2168,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2087,7 +2195,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2114,7 +2222,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2141,7 +2249,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2168,7 +2276,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2195,7 +2303,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2222,7 +2330,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2249,7 +2357,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2276,7 +2384,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2303,7 +2411,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2330,7 +2438,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2357,7 +2465,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -2369,6 +2477,33 @@
         <ser>
           <idx val="12"/>
           <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2387,39 +2522,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$3</f>
             </numRef>
           </val>
         </ser>
@@ -2441,12 +2549,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2468,12 +2576,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2495,12 +2603,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2522,12 +2630,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2549,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2576,12 +2684,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2603,12 +2711,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2630,12 +2738,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2765,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -2684,12 +2792,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -2711,18 +2819,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="25"/>
           <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2741,66 +2903,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="26"/>
-          <order val="26"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="27"/>
-          <order val="27"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$4</f>
             </numRef>
           </val>
         </ser>
@@ -2822,12 +2930,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2849,12 +2957,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2876,12 +2984,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2903,12 +3011,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2930,12 +3038,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2957,12 +3065,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -2984,12 +3092,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -3011,12 +3119,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -3038,12 +3146,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -3065,18 +3173,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="38"/>
           <order val="38"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="39"/>
+          <order val="39"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="41"/>
+          <order val="41"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -3095,93 +3284,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="39"/>
-          <order val="39"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="40"/>
-          <order val="40"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="41"/>
-          <order val="41"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$5</f>
             </numRef>
           </val>
         </ser>
@@ -3203,12 +3311,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -3230,12 +3338,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -3257,12 +3365,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -3284,12 +3392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -3311,12 +3419,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -3338,12 +3446,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -3365,12 +3473,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3392,12 +3500,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -3419,18 +3527,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="51"/>
           <order val="51"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="52"/>
+          <order val="52"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="53"/>
+          <order val="53"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="54"/>
+          <order val="54"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="55"/>
+          <order val="55"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -3449,120 +3665,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="52"/>
-          <order val="52"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="53"/>
-          <order val="53"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="54"/>
-          <order val="54"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="55"/>
-          <order val="55"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$6</f>
             </numRef>
           </val>
         </ser>
@@ -3584,12 +3692,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -3611,12 +3719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -3638,12 +3746,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -3665,12 +3773,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -3692,12 +3800,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -3719,12 +3827,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
@@ -3746,12 +3854,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -3773,18 +3881,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="64"/>
           <order val="64"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="65"/>
+          <order val="65"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="66"/>
+          <order val="66"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="67"/>
+          <order val="67"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="68"/>
+          <order val="68"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="69"/>
+          <order val="69"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -3803,12 +4046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$7</f>
             </numRef>
           </val>
         </ser>
@@ -3917,7 +4160,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -3944,7 +4187,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -3971,7 +4214,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -3998,7 +4241,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4025,7 +4268,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4052,7 +4295,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4079,7 +4322,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4106,7 +4349,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4133,7 +4376,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4160,7 +4403,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4187,7 +4430,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4214,7 +4457,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
             </numRef>
           </cat>
           <val>
@@ -4226,6 +4469,33 @@
         <ser>
           <idx val="12"/>
           <order val="12"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -4244,39 +4514,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$N$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$3</f>
             </numRef>
           </val>
         </ser>
@@ -4298,12 +4541,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -4325,12 +4568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -4352,12 +4595,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -4379,12 +4622,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -4406,12 +4649,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -4433,12 +4676,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -4460,12 +4703,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -4487,12 +4730,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -4514,12 +4757,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -4541,12 +4784,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -4568,18 +4811,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="25"/>
           <order val="25"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -4598,12 +4895,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$N$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$N$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$4</f>
             </numRef>
           </val>
         </ser>
@@ -4678,7 +4975,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -5089,14 +5386,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 06/06/2026 11:16</t>
+          <t>Última actualización: 07/06/2026 12:12</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-06</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5445,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-06</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5517,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-06</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5530,6 +5827,22 @@
         <v>17.64</v>
       </c>
       <c r="D15" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D16" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -5548,7 +5861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5565,6 +5878,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5643,6 +5957,11 @@
       <c r="N2" s="24" t="inlineStr">
         <is>
           <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="O2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
         </is>
       </c>
     </row>
@@ -5673,6 +5992,7 @@
       <c r="L3" s="19" t="n"/>
       <c r="M3" s="19" t="n"/>
       <c r="N3" s="19" t="n"/>
+      <c r="O3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5713,6 +6033,7 @@
       <c r="L4" s="21" t="n"/>
       <c r="M4" s="21" t="n"/>
       <c r="N4" s="21" t="n"/>
+      <c r="O4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -5753,6 +6074,9 @@
       <c r="N5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="O5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -5797,10 +6121,13 @@
       <c r="N6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="O6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5813,7 +6140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5830,6 +6157,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5910,6 +6238,11 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="O2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -5950,6 +6283,7 @@
       <c r="L3" s="19" t="n"/>
       <c r="M3" s="19" t="n"/>
       <c r="N3" s="19" t="n"/>
+      <c r="O3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -5994,6 +6328,9 @@
         <v>16.84</v>
       </c>
       <c r="N4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="O4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -6036,6 +6373,9 @@
       <c r="N5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="O5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6080,6 +6420,9 @@
         <v>17.99</v>
       </c>
       <c r="N6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="O6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -6114,10 +6457,13 @@
       <c r="N7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="O7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6130,7 +6476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6147,6 +6493,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6227,6 +6574,11 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="O2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -6273,6 +6625,9 @@
       <c r="N3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="O3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6319,10 +6674,13 @@
       <c r="N4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="O4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6335,7 +6693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F287"/>
+  <dimension ref="A1:F310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13504,6 +13862,581 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B288" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C288" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D288" s="21" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E288" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B289" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C289" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D289" s="19" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E289" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B290" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C290" s="33" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D290" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E290" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B291" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C291" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D291" s="19" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E291" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B292" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C292" s="33" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D292" s="21" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E292" s="33" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B293" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C293" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D293" s="19" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E293" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B294" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C294" s="33" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D294" s="21" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E294" s="33" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B295" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C295" s="32" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D295" s="19" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E295" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B296" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C296" s="33" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D296" s="21" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E296" s="33" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B297" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C297" s="32" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D297" s="19" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E297" s="32" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B298" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C298" s="33" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D298" s="21" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E298" s="33" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B299" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C299" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D299" s="19" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E299" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B300" s="33" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C300" s="33" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D300" s="21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E300" s="33" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B301" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C301" s="32" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D301" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="E301" s="32" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B302" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C302" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D302" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E302" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B303" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C303" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D303" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E303" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B304" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C304" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D304" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E304" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B305" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C305" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D305" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E305" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B306" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C306" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D306" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E306" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B307" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C307" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D307" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E307" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B308" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C308" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D308" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E308" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B309" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C309" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D309" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E309" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B310" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C310" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D310" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E310" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-08
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$16</f>
+              <f>'📊 Media diaria'!$A$3:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$17</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$16</f>
+              <f>'📊 Media diaria'!$A$3:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$17</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$16</f>
+              <f>'📊 Media diaria'!$A$3:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -827,7 +827,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -854,7 +854,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -881,7 +881,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -893,6 +893,33 @@
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -911,39 +938,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$3</f>
             </numRef>
           </val>
         </ser>
@@ -965,12 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1127,12 +1127,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1154,12 +1154,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1181,12 +1181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1208,12 +1208,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -1235,12 +1235,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -1262,18 +1262,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="27"/>
           <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1292,66 +1346,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="28"/>
-          <order val="28"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="29"/>
-          <order val="29"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$4</f>
             </numRef>
           </val>
         </ser>
@@ -1373,12 +1373,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1400,12 +1400,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1427,12 +1427,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1454,12 +1454,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1481,12 +1481,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1508,12 +1508,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1535,12 +1535,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1562,12 +1562,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1589,12 +1589,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -1616,12 +1616,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -1643,18 +1643,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="41"/>
           <order val="41"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="42"/>
+          <order val="42"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="43"/>
+          <order val="43"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="44"/>
+          <order val="44"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1673,93 +1754,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="42"/>
-          <order val="42"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="43"/>
-          <order val="43"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="44"/>
-          <order val="44"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$5</f>
             </numRef>
           </val>
         </ser>
@@ -1781,12 +1781,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1808,12 +1808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1835,12 +1835,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1862,12 +1862,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1889,12 +1889,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1916,12 +1916,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1943,12 +1943,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1970,12 +1970,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1997,12 +1997,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -2024,18 +2024,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="55"/>
           <order val="55"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="56"/>
+          <order val="56"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="57"/>
+          <order val="57"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="58"/>
+          <order val="58"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="59"/>
+          <order val="59"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -2054,12 +2162,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$6</f>
             </numRef>
           </val>
         </ser>
@@ -2168,7 +2276,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2195,7 +2303,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2222,7 +2330,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2249,7 +2357,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2276,7 +2384,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2303,7 +2411,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2330,7 +2438,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2357,7 +2465,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2384,7 +2492,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2411,7 +2519,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2438,7 +2546,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2465,7 +2573,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2492,7 +2600,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -2504,6 +2612,33 @@
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2522,39 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$3</f>
             </numRef>
           </val>
         </ser>
@@ -2576,12 +2684,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2603,12 +2711,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2630,12 +2738,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2765,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2684,12 +2792,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2711,12 +2819,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2738,12 +2846,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2765,12 +2873,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2792,12 +2900,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -2819,12 +2927,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -2846,12 +2954,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -2873,18 +2981,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="27"/>
           <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -2903,66 +3065,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="28"/>
-          <order val="28"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="29"/>
-          <order val="29"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$4</f>
             </numRef>
           </val>
         </ser>
@@ -2984,12 +3092,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -3011,12 +3119,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -3038,12 +3146,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -3065,12 +3173,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -3092,12 +3200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -3119,12 +3227,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -3146,12 +3254,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -3173,12 +3281,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -3200,12 +3308,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -3227,12 +3335,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -3254,18 +3362,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="41"/>
           <order val="41"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="42"/>
+          <order val="42"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="43"/>
+          <order val="43"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="44"/>
+          <order val="44"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -3284,93 +3473,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="42"/>
-          <order val="42"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="43"/>
-          <order val="43"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="44"/>
-          <order val="44"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$5</f>
             </numRef>
           </val>
         </ser>
@@ -3392,12 +3500,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -3419,12 +3527,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -3446,12 +3554,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -3473,12 +3581,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -3500,12 +3608,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -3527,12 +3635,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -3554,12 +3662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3581,12 +3689,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -3608,12 +3716,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -3635,18 +3743,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="55"/>
           <order val="55"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="56"/>
+          <order val="56"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="57"/>
+          <order val="57"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="58"/>
+          <order val="58"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="59"/>
+          <order val="59"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -3665,120 +3881,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="56"/>
-          <order val="56"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="57"/>
-          <order val="57"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="58"/>
-          <order val="58"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="59"/>
-          <order val="59"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$6</f>
             </numRef>
           </val>
         </ser>
@@ -3800,12 +3908,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -3827,12 +3935,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -3854,12 +3962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -3881,12 +3989,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -3908,12 +4016,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -3935,12 +4043,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
@@ -3962,12 +4070,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -3989,12 +4097,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -4016,18 +4124,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="69"/>
           <order val="69"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="70"/>
+          <order val="70"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="71"/>
+          <order val="71"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="72"/>
+          <order val="72"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="73"/>
+          <order val="73"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="74"/>
+          <order val="74"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -4046,12 +4289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$7</f>
             </numRef>
           </val>
         </ser>
@@ -4160,7 +4403,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4187,7 +4430,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4214,7 +4457,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4241,7 +4484,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4268,7 +4511,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4295,7 +4538,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4322,7 +4565,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4349,7 +4592,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4376,7 +4619,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4403,7 +4646,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4430,7 +4673,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4457,7 +4700,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4484,7 +4727,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
             </numRef>
           </cat>
           <val>
@@ -4496,6 +4739,33 @@
         <ser>
           <idx val="13"/>
           <order val="13"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -4514,39 +4784,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$O$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$P$3</f>
             </numRef>
           </val>
         </ser>
@@ -4568,12 +4811,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -4595,12 +4838,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -4622,12 +4865,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -4649,12 +4892,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -4676,12 +4919,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -4703,12 +4946,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -4730,12 +4973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -4757,12 +5000,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -4784,12 +5027,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -4811,12 +5054,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -4838,12 +5081,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -4865,18 +5108,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$N$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="27"/>
           <order val="27"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -4895,12 +5192,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$O$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$O$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$P$4</f>
             </numRef>
           </val>
         </ser>
@@ -4975,7 +5272,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -5386,14 +5683,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 07/06/2026 12:12</t>
+          <t>Última actualización: 08/06/2026 17:41</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-07</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -5445,7 +5742,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-07</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -5517,7 +5814,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-07</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5843,6 +6140,22 @@
         <v>17.64</v>
       </c>
       <c r="D16" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D17" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -5861,7 +6174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5879,6 +6192,7 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5962,6 +6276,11 @@
       <c r="O2" s="24" t="inlineStr">
         <is>
           <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -5993,6 +6312,7 @@
       <c r="M3" s="19" t="n"/>
       <c r="N3" s="19" t="n"/>
       <c r="O3" s="19" t="n"/>
+      <c r="P3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6034,6 +6354,7 @@
       <c r="M4" s="21" t="n"/>
       <c r="N4" s="21" t="n"/>
       <c r="O4" s="21" t="n"/>
+      <c r="P4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -6077,6 +6398,9 @@
       <c r="O5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="P5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6124,10 +6448,13 @@
       <c r="O6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="P6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6140,7 +6467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6158,6 +6485,7 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6243,6 +6571,11 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="P2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -6284,6 +6617,7 @@
       <c r="M3" s="19" t="n"/>
       <c r="N3" s="19" t="n"/>
       <c r="O3" s="19" t="n"/>
+      <c r="P3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6331,6 +6665,9 @@
         <v>16.84</v>
       </c>
       <c r="O4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="P4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -6376,6 +6713,9 @@
       <c r="O5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="P5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6423,6 +6763,9 @@
         <v>17.99</v>
       </c>
       <c r="O6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="P6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -6460,10 +6803,13 @@
       <c r="O7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="P7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6476,7 +6822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6494,6 +6840,7 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6579,6 +6926,11 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="P2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -6628,6 +6980,9 @@
       <c r="O3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="P3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6677,10 +7032,13 @@
       <c r="O4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="P4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6693,7 +7051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F310"/>
+  <dimension ref="A1:F334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14437,6 +14795,606 @@
         </is>
       </c>
     </row>
+    <row r="311">
+      <c r="A311" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B311" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C311" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D311" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E311" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B312" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C312" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D312" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E312" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B313" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C313" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D313" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E313" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B314" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C314" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D314" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E314" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B315" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C315" s="32" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D315" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E315" s="32" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B316" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C316" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D316" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E316" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B317" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C317" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D317" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E317" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B318" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C318" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D318" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E318" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B319" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C319" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D319" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E319" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B320" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C320" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D320" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E320" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B321" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C321" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D321" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E321" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B322" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C322" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D322" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E322" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B323" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C323" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D323" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E323" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B324" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C324" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D324" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E324" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B325" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C325" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D325" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E325" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B326" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C326" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D326" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E326" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B327" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C327" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D327" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E327" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B328" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C328" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D328" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E328" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B329" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C329" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D329" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E329" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B330" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C330" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D330" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E330" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B331" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C331" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D331" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E331" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B332" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C332" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D332" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E332" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B333" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C333" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D333" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E333" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B334" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C334" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D334" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E334" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-09
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$17</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$17</f>
+              <f>'📊 Media diaria'!$A$3:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$18</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$17</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$17</f>
+              <f>'📊 Media diaria'!$A$3:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$18</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$17</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$17</f>
+              <f>'📊 Media diaria'!$A$3:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$18</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -827,7 +827,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -854,7 +854,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -881,7 +881,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -908,7 +908,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -920,6 +920,33 @@
         <ser>
           <idx val="14"/>
           <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -938,39 +965,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$3</f>
             </numRef>
           </val>
         </ser>
@@ -992,12 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1127,12 +1127,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1154,12 +1154,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1181,12 +1181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1208,12 +1208,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1235,12 +1235,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -1262,12 +1262,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -1289,12 +1289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -1316,18 +1316,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="29"/>
           <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1346,66 +1400,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="30"/>
-          <order val="30"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="31"/>
-          <order val="31"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$4</f>
             </numRef>
           </val>
         </ser>
@@ -1427,12 +1427,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1454,12 +1454,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1481,12 +1481,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1508,12 +1508,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1535,12 +1535,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1562,12 +1562,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1589,12 +1589,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1616,12 +1616,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1643,12 +1643,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -1670,12 +1670,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -1697,12 +1697,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -1724,18 +1724,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="44"/>
           <order val="44"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="45"/>
+          <order val="45"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="46"/>
+          <order val="46"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="47"/>
+          <order val="47"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1754,93 +1835,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="45"/>
-          <order val="45"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="46"/>
-          <order val="46"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="47"/>
-          <order val="47"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$5</f>
             </numRef>
           </val>
         </ser>
@@ -1862,12 +1862,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1889,12 +1889,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1916,12 +1916,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1943,12 +1943,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1970,12 +1970,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -1997,12 +1997,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -2024,12 +2024,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2051,12 +2051,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2078,12 +2078,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -2105,12 +2105,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -2132,18 +2132,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="59"/>
           <order val="59"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="60"/>
+          <order val="60"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="61"/>
+          <order val="61"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="62"/>
+          <order val="62"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="63"/>
+          <order val="63"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -2162,12 +2270,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$6</f>
             </numRef>
           </val>
         </ser>
@@ -2276,7 +2384,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2303,7 +2411,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2330,7 +2438,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2357,7 +2465,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2384,7 +2492,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2411,7 +2519,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2438,7 +2546,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2465,7 +2573,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2492,7 +2600,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2519,7 +2627,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2546,7 +2654,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2573,7 +2681,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2600,7 +2708,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2627,7 +2735,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -2639,6 +2747,33 @@
         <ser>
           <idx val="14"/>
           <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2657,39 +2792,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$3</f>
             </numRef>
           </val>
         </ser>
@@ -2711,12 +2819,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2738,12 +2846,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2765,12 +2873,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2792,12 +2900,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2819,12 +2927,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2846,12 +2954,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -2873,12 +2981,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2900,12 +3008,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2927,12 +3035,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -2954,12 +3062,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -2981,12 +3089,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -3008,12 +3116,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -3035,18 +3143,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="29"/>
           <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -3065,66 +3227,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="30"/>
-          <order val="30"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="31"/>
-          <order val="31"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$4</f>
             </numRef>
           </val>
         </ser>
@@ -3146,12 +3254,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -3173,12 +3281,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -3200,12 +3308,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -3227,12 +3335,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -3254,12 +3362,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -3281,12 +3389,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -3308,12 +3416,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -3335,12 +3443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -3362,12 +3470,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -3389,12 +3497,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -3416,12 +3524,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -3443,18 +3551,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="44"/>
           <order val="44"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="45"/>
+          <order val="45"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="46"/>
+          <order val="46"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="47"/>
+          <order val="47"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -3473,93 +3662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="45"/>
-          <order val="45"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="46"/>
-          <order val="46"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="47"/>
-          <order val="47"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$5</f>
             </numRef>
           </val>
         </ser>
@@ -3581,12 +3689,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -3608,12 +3716,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -3635,12 +3743,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -3662,12 +3770,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -3689,12 +3797,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -3716,12 +3824,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -3743,12 +3851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3770,12 +3878,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -3797,12 +3905,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -3824,12 +3932,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -3851,18 +3959,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="59"/>
           <order val="59"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="60"/>
+          <order val="60"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="61"/>
+          <order val="61"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="62"/>
+          <order val="62"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="63"/>
+          <order val="63"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -3881,120 +4097,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="60"/>
-          <order val="60"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="61"/>
-          <order val="61"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="62"/>
-          <order val="62"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="63"/>
-          <order val="63"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$6</f>
             </numRef>
           </val>
         </ser>
@@ -4016,12 +4124,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -4043,12 +4151,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -4070,12 +4178,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -4097,12 +4205,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -4124,12 +4232,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -4151,12 +4259,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
@@ -4178,12 +4286,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -4205,12 +4313,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -4232,12 +4340,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
             </numRef>
           </val>
         </ser>
@@ -4259,18 +4367,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="74"/>
           <order val="74"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="75"/>
+          <order val="75"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="76"/>
+          <order val="76"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="77"/>
+          <order val="77"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="78"/>
+          <order val="78"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="79"/>
+          <order val="79"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -4289,12 +4532,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$7</f>
             </numRef>
           </val>
         </ser>
@@ -4403,7 +4646,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4430,7 +4673,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4457,7 +4700,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4484,7 +4727,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4511,7 +4754,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4538,7 +4781,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4565,7 +4808,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4592,7 +4835,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4619,7 +4862,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4646,7 +4889,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4673,7 +4916,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4700,7 +4943,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4727,7 +4970,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4754,7 +4997,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
             </numRef>
           </cat>
           <val>
@@ -4766,6 +5009,33 @@
         <ser>
           <idx val="14"/>
           <order val="14"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$P$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -4784,39 +5054,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$P$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$Q$3</f>
             </numRef>
           </val>
         </ser>
@@ -4838,12 +5081,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -4865,12 +5108,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -4892,12 +5135,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -4919,12 +5162,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -4946,12 +5189,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -4973,12 +5216,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -5000,12 +5243,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -5027,12 +5270,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -5054,12 +5297,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -5081,12 +5324,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -5108,12 +5351,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -5135,12 +5378,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$N$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -5162,18 +5405,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$O$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="29"/>
           <order val="29"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -5192,12 +5489,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$P$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$P$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$Q$4</f>
             </numRef>
           </val>
         </ser>
@@ -5272,7 +5569,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -5683,14 +5980,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 08/06/2026 17:41</t>
+          <t>Última actualización: 09/06/2026 16:23</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-08</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -5742,7 +6039,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-08</t>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -5814,7 +6111,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-08</t>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -5881,7 +6178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6156,6 +6453,22 @@
         <v>17.64</v>
       </c>
       <c r="D17" s="19" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D18" s="21" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -6174,7 +6487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6193,6 +6506,7 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6281,6 +6595,11 @@
       <c r="P2" s="24" t="inlineStr">
         <is>
           <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="Q2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -6313,6 +6632,7 @@
       <c r="N3" s="19" t="n"/>
       <c r="O3" s="19" t="n"/>
       <c r="P3" s="19" t="n"/>
+      <c r="Q3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6355,6 +6675,7 @@
       <c r="N4" s="21" t="n"/>
       <c r="O4" s="21" t="n"/>
       <c r="P4" s="21" t="n"/>
+      <c r="Q4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -6401,6 +6722,9 @@
       <c r="P5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="Q5" s="19" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6451,10 +6775,13 @@
       <c r="P6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="Q6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6467,7 +6794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6486,6 +6813,7 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6574,6 +6902,11 @@
       <c r="P2" s="28" t="inlineStr">
         <is>
           <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="Q2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -6618,6 +6951,7 @@
       <c r="N3" s="19" t="n"/>
       <c r="O3" s="19" t="n"/>
       <c r="P3" s="19" t="n"/>
+      <c r="Q3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6668,6 +7002,9 @@
         <v>16.84</v>
       </c>
       <c r="P4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="Q4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -6716,6 +7053,9 @@
       <c r="P5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="Q5" s="19" t="n">
+        <v>18.87</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6766,6 +7106,9 @@
         <v>17.99</v>
       </c>
       <c r="P6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="Q6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -6806,10 +7149,13 @@
       <c r="P7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="Q7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6822,7 +7168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6841,6 +7187,7 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6931,6 +7278,11 @@
           <t>2026-06-08</t>
         </is>
       </c>
+      <c r="Q2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -6983,6 +7335,9 @@
       <c r="P3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="Q3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -7035,10 +7390,13 @@
       <c r="P4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="Q4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7051,7 +7409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F334"/>
+  <dimension ref="A1:F358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15395,6 +15753,606 @@
         </is>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B335" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C335" s="32" t="inlineStr">
+        <is>
+          <t>Madrid Camper 522</t>
+        </is>
+      </c>
+      <c r="D335" s="19" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E335" s="32" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9522-sikaflex-522-blanco.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B336" s="33" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C336" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D336" s="21" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E336" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B337" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C337" s="32" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D337" s="19" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E337" s="32" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B338" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C338" s="33" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D338" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E338" s="33" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B339" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C339" s="32" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D339" s="19" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E339" s="32" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B340" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C340" s="33" t="inlineStr">
+        <is>
+          <t>Madrid Camper 554</t>
+        </is>
+      </c>
+      <c r="D340" s="21" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="E340" s="33" t="inlineStr">
+        <is>
+          <t>https://madridcamper.com/selladores-y-adhesivos/9519-sikaflex-554-negro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B341" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C341" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D341" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E341" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B342" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C342" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D342" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E342" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B343" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C343" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D343" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E343" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B344" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C344" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D344" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E344" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B345" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C345" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D345" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E345" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B346" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C346" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D346" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E346" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B347" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C347" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D347" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E347" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B348" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C348" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D348" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E348" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B349" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C349" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D349" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E349" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B350" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C350" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D350" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E350" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B351" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C351" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D351" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E351" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B352" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C352" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D352" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E352" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B353" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C353" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D353" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E353" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B354" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C354" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D354" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E354" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B355" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C355" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D355" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E355" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B356" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C356" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D356" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E356" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B357" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C357" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D357" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E357" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B358" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C358" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D358" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E358" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
📊 Precios actualizados 2026-06-10
</commit_message>
<xml_diff>
--- a/precios_sikaflex.xlsx
+++ b/precios_sikaflex.xlsx
@@ -174,16 +174,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -371,12 +371,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$18</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$B$3:$B$18</f>
+              <f>'📊 Media diaria'!$A$3:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$B$3:$B$19</f>
             </numRef>
           </val>
         </ser>
@@ -407,12 +407,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$18</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$C$3:$C$18</f>
+              <f>'📊 Media diaria'!$A$3:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$C$3:$C$19</f>
             </numRef>
           </val>
         </ser>
@@ -443,12 +443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'📊 Media diaria'!$A$3:$A$18</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Media diaria'!$D$3:$D$18</f>
+              <f>'📊 Media diaria'!$A$3:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'📊 Media diaria'!$D$3:$D$19</f>
             </numRef>
           </val>
         </ser>
@@ -557,7 +557,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -584,7 +584,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -611,7 +611,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -638,7 +638,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -665,7 +665,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -692,7 +692,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -719,7 +719,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -746,7 +746,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -773,7 +773,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -800,7 +800,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -827,7 +827,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -854,7 +854,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -881,7 +881,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -908,7 +908,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -935,7 +935,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -947,6 +947,33 @@
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
           <tx>
             <v>Andorra Campers</v>
           </tx>
@@ -965,39 +992,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$Q$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$R$3</f>
             </numRef>
           </val>
         </ser>
@@ -1019,12 +1019,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1046,12 +1046,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -1073,12 +1073,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1127,12 +1127,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -1154,12 +1154,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1181,12 +1181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1208,12 +1208,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1235,12 +1235,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -1262,12 +1262,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -1289,12 +1289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -1316,12 +1316,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -1343,12 +1343,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -1370,18 +1370,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$4</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="31"/>
           <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
           <tx>
             <v>Barna Campers</v>
           </tx>
@@ -1400,66 +1454,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$Q$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="32"/>
-          <order val="32"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="33"/>
-          <order val="33"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$R$4</f>
             </numRef>
           </val>
         </ser>
@@ -1481,12 +1481,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -1508,12 +1508,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1535,12 +1535,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1562,12 +1562,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1589,12 +1589,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -1616,12 +1616,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1643,12 +1643,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1670,12 +1670,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1697,12 +1697,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -1724,12 +1724,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -1778,12 +1778,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$5</f>
             </numRef>
           </val>
         </ser>
@@ -1805,18 +1805,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$5</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="47"/>
           <order val="47"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="48"/>
+          <order val="48"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="49"/>
+          <order val="49"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="50"/>
+          <order val="50"/>
           <tx>
             <v>Madrid Camper 522</v>
           </tx>
@@ -1835,93 +1916,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$Q$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="48"/>
-          <order val="48"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="49"/>
-          <order val="49"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="50"/>
-          <order val="50"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$D$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$R$5</f>
             </numRef>
           </val>
         </ser>
@@ -1943,12 +1943,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$E$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1970,12 +1970,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$F$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -1997,12 +1997,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$G$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2024,12 +2024,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$H$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2051,12 +2051,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$I$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -2078,12 +2078,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$J$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -2105,12 +2105,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$K$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2132,12 +2132,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$L$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2159,12 +2159,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$M$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -2186,12 +2186,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$N$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -2213,12 +2213,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$O$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$L$6</f>
             </numRef>
           </val>
         </ser>
@@ -2240,18 +2240,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$P$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$M$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="63"/>
           <order val="63"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="64"/>
+          <order val="64"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="65"/>
+          <order val="65"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$P$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="66"/>
+          <order val="66"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$Q$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="67"/>
+          <order val="67"/>
           <tx>
             <v>Obelink 522</v>
           </tx>
@@ -2270,12 +2378,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🔵 Sikaflex 522'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🔵 Sikaflex 522'!$Q$6</f>
+              <f>'🔵 Sikaflex 522'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🔵 Sikaflex 522'!$R$6</f>
             </numRef>
           </val>
         </ser>
@@ -2384,7 +2492,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2411,7 +2519,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2438,7 +2546,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2465,7 +2573,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2492,7 +2600,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2519,7 +2627,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2546,7 +2654,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2573,7 +2681,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2600,7 +2708,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2627,7 +2735,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2654,7 +2762,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2681,7 +2789,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2708,7 +2816,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2735,7 +2843,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2762,7 +2870,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -2774,6 +2882,33 @@
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
           <tx>
             <v>Berger Camping 554</v>
           </tx>
@@ -2792,39 +2927,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$Q$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$R$3</f>
             </numRef>
           </val>
         </ser>
@@ -2846,12 +2954,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -2873,12 +2981,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -2900,12 +3008,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2927,12 +3035,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2954,12 +3062,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -2981,12 +3089,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -3008,12 +3116,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -3035,12 +3143,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -3062,12 +3170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -3089,12 +3197,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -3116,12 +3224,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -3143,12 +3251,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -3170,12 +3278,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -3197,18 +3305,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$4</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="31"/>
           <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
           <tx>
             <v>Intercut 554</v>
           </tx>
@@ -3227,66 +3389,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$Q$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="32"/>
-          <order val="32"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="33"/>
-          <order val="33"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$R$4</f>
             </numRef>
           </val>
         </ser>
@@ -3308,12 +3416,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -3335,12 +3443,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -3362,12 +3470,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -3389,12 +3497,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -3416,12 +3524,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -3443,12 +3551,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -3470,12 +3578,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -3497,12 +3605,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -3524,12 +3632,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$5</f>
             </numRef>
           </val>
         </ser>
@@ -3551,12 +3659,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$5</f>
             </numRef>
           </val>
         </ser>
@@ -3578,12 +3686,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$5</f>
             </numRef>
           </val>
         </ser>
@@ -3605,12 +3713,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$5</f>
             </numRef>
           </val>
         </ser>
@@ -3632,18 +3740,99 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$5</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$5</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="47"/>
           <order val="47"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="48"/>
+          <order val="48"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="49"/>
+          <order val="49"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="50"/>
+          <order val="50"/>
           <tx>
             <v>Madrid Camper 554</v>
           </tx>
@@ -3662,93 +3851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$Q$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="48"/>
-          <order val="48"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="49"/>
-          <order val="49"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="50"/>
-          <order val="50"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$R$5</f>
             </numRef>
           </val>
         </ser>
@@ -3770,12 +3878,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -3797,12 +3905,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -3824,12 +3932,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -3851,12 +3959,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -3878,12 +3986,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -3905,12 +4013,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -3932,12 +4040,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3959,12 +4067,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -3986,12 +4094,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -4013,12 +4121,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$6</f>
             </numRef>
           </val>
         </ser>
@@ -4040,12 +4148,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$6</f>
             </numRef>
           </val>
         </ser>
@@ -4067,18 +4175,126 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$6</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$6</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="63"/>
           <order val="63"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="64"/>
+          <order val="64"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="65"/>
+          <order val="65"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="66"/>
+          <order val="66"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="67"/>
+          <order val="67"/>
           <tx>
             <v>Obelink 554</v>
           </tx>
@@ -4097,120 +4313,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$Q$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="64"/>
-          <order val="64"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="65"/>
-          <order val="65"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$C$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="66"/>
-          <order val="66"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$D$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="67"/>
-          <order val="67"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$E$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$R$6</f>
             </numRef>
           </val>
         </ser>
@@ -4232,12 +4340,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$F$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -4259,12 +4367,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$G$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -4286,12 +4394,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$H$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -4313,12 +4421,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$I$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -4340,12 +4448,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$J$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -4367,12 +4475,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$K$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$G$7</f>
             </numRef>
           </val>
         </ser>
@@ -4394,12 +4502,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$L$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -4421,12 +4529,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$M$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -4448,12 +4556,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$N$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$J$7</f>
             </numRef>
           </val>
         </ser>
@@ -4475,12 +4583,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$O$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$K$7</f>
             </numRef>
           </val>
         </ser>
@@ -4502,18 +4610,153 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$P$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$L$7</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="79"/>
           <order val="79"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$M$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="80"/>
+          <order val="80"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$N$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="81"/>
+          <order val="81"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$O$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="82"/>
+          <order val="82"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$P$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="83"/>
+          <order val="83"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$Q$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="84"/>
+          <order val="84"/>
           <tx>
             <v>TodoCampers 554</v>
           </tx>
@@ -4532,12 +4775,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟣 Sikaflex 554'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟣 Sikaflex 554'!$Q$7</f>
+              <f>'🟣 Sikaflex 554'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟣 Sikaflex 554'!$R$7</f>
             </numRef>
           </val>
         </ser>
@@ -4646,7 +4889,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4673,7 +4916,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4700,7 +4943,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4727,7 +4970,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4754,7 +4997,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4781,7 +5024,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4808,7 +5051,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4835,7 +5078,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4862,7 +5105,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4889,7 +5132,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4916,7 +5159,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4943,7 +5186,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4970,7 +5213,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -4997,7 +5240,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -5024,7 +5267,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
             </numRef>
           </cat>
           <val>
@@ -5036,6 +5279,33 @@
         <ser>
           <idx val="15"/>
           <order val="15"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$Q$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
           <tx>
             <v>Plana Online 621</v>
           </tx>
@@ -5054,39 +5324,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$Q$3</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$B$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$R$3</f>
             </numRef>
           </val>
         </ser>
@@ -5108,12 +5351,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$C$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -5135,12 +5378,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$D$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$C$4</f>
             </numRef>
           </val>
         </ser>
@@ -5162,12 +5405,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$E$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -5189,12 +5432,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$F$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -5216,12 +5459,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$G$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -5243,12 +5486,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$H$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -5270,12 +5513,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$I$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -5297,12 +5540,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$J$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -5324,12 +5567,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$K$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$J$4</f>
             </numRef>
           </val>
         </ser>
@@ -5351,12 +5594,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$L$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$K$4</f>
             </numRef>
           </val>
         </ser>
@@ -5378,12 +5621,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$M$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$L$4</f>
             </numRef>
           </val>
         </ser>
@@ -5405,12 +5648,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$N$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$M$4</f>
             </numRef>
           </val>
         </ser>
@@ -5432,12 +5675,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$O$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$N$4</f>
             </numRef>
           </val>
         </ser>
@@ -5459,18 +5702,72 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$P$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$O$4</f>
             </numRef>
           </val>
         </ser>
         <ser>
           <idx val="31"/>
           <order val="31"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$P$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$Q$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
           <tx>
             <v>Toolstock 621</v>
           </tx>
@@ -5489,12 +5786,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🟢 Sikaflex 621'!$B$2:$Q$2</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'🟢 Sikaflex 621'!$Q$4</f>
+              <f>'🟢 Sikaflex 621'!$B$2:$R$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'🟢 Sikaflex 621'!$R$4</f>
             </numRef>
           </val>
         </ser>
@@ -5569,7 +5866,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -5960,7 +6257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5980,14 +6277,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 09/06/2026 16:23</t>
+          <t>Última actualización: 10/06/2026 17:48</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-09</t>
+          <t xml:space="preserve">  SIKAFLEX 522 — Precios del 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -6021,140 +6318,115 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 522</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>🔴 Más caro</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 554 — Precios del 2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>✅ Más barato</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Intercut 554</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>✅ Más barato</t>
-        </is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>16.85</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>TodoCampers 554</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n">
-        <v>16.85</v>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
           <t>Obelink 554</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <v>17.99</v>
       </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Madrid Camper 554</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>18.87</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIKAFLEX 621 — Precios del 2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Plana Online 621</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B16" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>✅ Más barato</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Toolstock 621</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B17" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>🔴 Más caro</t>
         </is>
@@ -6164,9 +6436,9 @@
   <mergeCells count="5">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6178,7 +6450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6469,6 +6741,22 @@
         <v>17.64</v>
       </c>
       <c r="D18" s="21" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="D19" s="19" t="n">
         <v>13.4</v>
       </c>
     </row>
@@ -6487,7 +6775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6507,6 +6795,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6600,6 +6889,11 @@
       <c r="Q2" s="24" t="inlineStr">
         <is>
           <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="R2" s="24" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -6633,6 +6927,7 @@
       <c r="O3" s="19" t="n"/>
       <c r="P3" s="19" t="n"/>
       <c r="Q3" s="19" t="n"/>
+      <c r="R3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -6676,6 +6971,7 @@
       <c r="O4" s="21" t="n"/>
       <c r="P4" s="21" t="n"/>
       <c r="Q4" s="21" t="n"/>
+      <c r="R4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -6725,6 +7021,7 @@
       <c r="Q5" s="19" t="n">
         <v>12.4</v>
       </c>
+      <c r="R5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -6778,10 +7075,13 @@
       <c r="Q6" s="21" t="n">
         <v>10.99</v>
       </c>
+      <c r="R6" s="21" t="n">
+        <v>10.99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6794,7 +7094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6814,6 +7114,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6907,6 +7208,11 @@
       <c r="Q2" s="28" t="inlineStr">
         <is>
           <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="R2" s="28" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -6952,6 +7258,7 @@
       <c r="O3" s="19" t="n"/>
       <c r="P3" s="19" t="n"/>
       <c r="Q3" s="19" t="n"/>
+      <c r="R3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -7005,6 +7312,9 @@
         <v>16.84</v>
       </c>
       <c r="Q4" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="R4" s="21" t="n">
         <v>16.84</v>
       </c>
     </row>
@@ -7056,6 +7366,7 @@
       <c r="Q5" s="19" t="n">
         <v>18.87</v>
       </c>
+      <c r="R5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -7109,6 +7420,9 @@
         <v>17.99</v>
       </c>
       <c r="Q6" s="21" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="R6" s="21" t="n">
         <v>17.99</v>
       </c>
     </row>
@@ -7152,10 +7466,13 @@
       <c r="Q7" s="19" t="n">
         <v>16.85</v>
       </c>
+      <c r="R7" s="19" t="n">
+        <v>16.85</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7168,7 +7485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7188,6 +7505,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7283,6 +7601,11 @@
           <t>2026-06-09</t>
         </is>
       </c>
+      <c r="R2" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -7338,6 +7661,9 @@
       <c r="Q3" s="19" t="n">
         <v>11.8</v>
       </c>
+      <c r="R3" s="19" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -7393,10 +7719,13 @@
       <c r="Q4" s="21" t="n">
         <v>15</v>
       </c>
+      <c r="R4" s="21" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7409,7 +7738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F358"/>
+  <dimension ref="A1:F380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16353,6 +16682,556 @@
         </is>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B359" s="32" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="C359" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 522</t>
+        </is>
+      </c>
+      <c r="D359" s="19" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="E359" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-522-kit-sellador-adhesivo-hibrido-white-628399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B360" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C360" s="33" t="inlineStr">
+        <is>
+          <t>Intercut 554</t>
+        </is>
+      </c>
+      <c r="D360" s="21" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="E360" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/sikaflex-554-300-ml-2284</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B361" s="32" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C361" s="32" t="inlineStr">
+        <is>
+          <t>Obelink 554</t>
+        </is>
+      </c>
+      <c r="D361" s="19" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="E361" s="32" t="inlineStr">
+        <is>
+          <t>https://www.obelink.es/sikaflex-554-kit-de-montaje-black-628401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B362" s="33" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="C362" s="33" t="inlineStr">
+        <is>
+          <t>TodoCampers 554</t>
+        </is>
+      </c>
+      <c r="D362" s="21" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="E362" s="33" t="inlineStr">
+        <is>
+          <t>https://todocampers.com/es/5041-sikaflex-554-negro-7612895736495.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B363" s="32" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C363" s="32" t="inlineStr">
+        <is>
+          <t>MasQueCamper T930</t>
+        </is>
+      </c>
+      <c r="D363" s="19" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="E363" s="32" t="inlineStr">
+        <is>
+          <t>https://www.masquecamper.com/producto/sellador-negro-terostat-ms-930-310-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B364" s="33" t="inlineStr">
+        <is>
+          <t>T930</t>
+        </is>
+      </c>
+      <c r="C364" s="33" t="inlineStr">
+        <is>
+          <t>Intercut T930</t>
+        </is>
+      </c>
+      <c r="D364" s="21" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="E364" s="33" t="inlineStr">
+        <is>
+          <t>https://intercut.es/products/teroson-ms-930-310ml-sellador-blanco-712</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B365" s="32" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C365" s="32" t="inlineStr">
+        <is>
+          <t>Diperplac BP795</t>
+        </is>
+      </c>
+      <c r="D365" s="19" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="E365" s="32" t="inlineStr">
+        <is>
+          <t>https://diperplac.com/tienda/colas-masillas-y-siliconas/3850-bostik-masilla-poliuretano-p795-flex-300ml-blanca.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B366" s="33" t="inlineStr">
+        <is>
+          <t>BP795</t>
+        </is>
+      </c>
+      <c r="C366" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Maquinaria BP795</t>
+        </is>
+      </c>
+      <c r="D366" s="21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E366" s="33" t="inlineStr">
+        <is>
+          <t>https://ferreteriaymaquinaria.com/producto/masilla-pu-bostik-p795-premium-cartucho-300-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B367" s="32" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C367" s="32" t="inlineStr">
+        <is>
+          <t>Aismar SF45</t>
+        </is>
+      </c>
+      <c r="D367" s="19" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="E367" s="32" t="inlineStr">
+        <is>
+          <t>https://www.poliuretanosaismar.com/tienda/resinas/reparacion-soudal/soudaflex-pu450-fc-300ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B368" s="33" t="inlineStr">
+        <is>
+          <t>SF45</t>
+        </is>
+      </c>
+      <c r="C368" s="33" t="inlineStr">
+        <is>
+          <t>Mengual SF45</t>
+        </is>
+      </c>
+      <c r="D368" s="21" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="E368" s="33" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/soudaflex-45fc-adhesivo-sellador-de-poliuretano</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B369" s="32" t="inlineStr">
+        <is>
+          <t>591</t>
+        </is>
+      </c>
+      <c r="C369" s="32" t="inlineStr">
+        <is>
+          <t>Netcoatings 591</t>
+        </is>
+      </c>
+      <c r="D369" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E369" s="32" t="inlineStr">
+        <is>
+          <t>https://netcoatings.shop/es/products/sikaflex-591-sellador-nautico-multiuso-pegamento-hibrido-para-barcos-sika-flex-blanco-300ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B370" s="33" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C370" s="33" t="inlineStr">
+        <is>
+          <t>GPS Nautico 291i</t>
+        </is>
+      </c>
+      <c r="D370" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E370" s="33" t="inlineStr">
+        <is>
+          <t>https://www.gpsnautico.com/es/accesorios-transductores/1684-sikaflex-291i-sellador-marino-300ml.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B371" s="32" t="inlineStr">
+        <is>
+          <t>291i</t>
+        </is>
+      </c>
+      <c r="C371" s="32" t="inlineStr">
+        <is>
+          <t>Naval Chicolino 291i</t>
+        </is>
+      </c>
+      <c r="D371" s="19" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E371" s="32" t="inlineStr">
+        <is>
+          <t>https://navalchicolino.com/producto/sikaflex-marino-291-blanco-o-negro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B372" s="33" t="inlineStr">
+        <is>
+          <t>3M5200</t>
+        </is>
+      </c>
+      <c r="C372" s="33" t="inlineStr">
+        <is>
+          <t>A.Alvarez 3M5200</t>
+        </is>
+      </c>
+      <c r="D372" s="21" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="E372" s="33" t="inlineStr">
+        <is>
+          <t>https://www.a-alvarez.com/51842-sellador-adhesivo-3m-secado-rapido-5200</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B373" s="32" t="inlineStr">
+        <is>
+          <t>3M4200</t>
+        </is>
+      </c>
+      <c r="C373" s="32" t="inlineStr">
+        <is>
+          <t>Shop-SKS 3M4200</t>
+        </is>
+      </c>
+      <c r="D373" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E373" s="32" t="inlineStr">
+        <is>
+          <t>https://www.shop-sks.com/es/3M-Adhesivo-y-sellador-de-poliuretano-marino-4200-FC-negro-310-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B374" s="33" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C374" s="33" t="inlineStr">
+        <is>
+          <t>Toolstock 621</t>
+        </is>
+      </c>
+      <c r="D374" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="E374" s="33" t="inlineStr">
+        <is>
+          <t>https://www.toolstock.info/principal/10201-SIKAFLEX-621CARTCH300CM3-NEGRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B375" s="32" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="C375" s="32" t="inlineStr">
+        <is>
+          <t>Plana Online 621</t>
+        </is>
+      </c>
+      <c r="D375" s="19" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E375" s="32" t="inlineStr">
+        <is>
+          <t>https://planaonline.com/es/nautica-y-marina/sikaflex-621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B376" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C376" s="33" t="inlineStr">
+        <is>
+          <t>Simor SS240</t>
+        </is>
+      </c>
+      <c r="D376" s="21" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E376" s="33" t="inlineStr">
+        <is>
+          <t>https://simor.es/producto/soudaseal-240-fc-290-ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B377" s="32" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C377" s="32" t="inlineStr">
+        <is>
+          <t>Mengual SS240</t>
+        </is>
+      </c>
+      <c r="D377" s="19" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E377" s="32" t="inlineStr">
+        <is>
+          <t>https://www.mengual.com/adhesivo-sellador-soudalseal-240fc-bolsa-de-600-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B378" s="33" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C378" s="33" t="inlineStr">
+        <is>
+          <t>Ferreteria Esmas QT</t>
+        </is>
+      </c>
+      <c r="D378" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E378" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ferreteriaesmas.com/adhesivos-de-montaje/117-polimero-adhesivo-fija-plus-turbo-quiadsa-8425608305791.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B379" s="32" t="inlineStr">
+        <is>
+          <t>QT</t>
+        </is>
+      </c>
+      <c r="C379" s="32" t="inlineStr">
+        <is>
+          <t>Destornillate QT</t>
+        </is>
+      </c>
+      <c r="D379" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E379" s="32" t="inlineStr">
+        <is>
+          <t>https://www.destornillate.es/producto/quiadsa-adhesivo-sellador-fija-plus-turbo-blanco-290ml/</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B380" s="33" t="inlineStr">
+        <is>
+          <t>SS240</t>
+        </is>
+      </c>
+      <c r="C380" s="33" t="inlineStr">
+        <is>
+          <t>Ventigo SS240</t>
+        </is>
+      </c>
+      <c r="D380" s="21" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="E380" s="33" t="inlineStr">
+        <is>
+          <t>https://www.ventigo.es/es_ES/p/sellador-adhesivo-ms-polimero-gris-soudaseal-240fc-tubo-290ml-unidad/5881/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>